<commit_message>
Lower Groq chunk size to 15000 to prevent 413 Too Large errors
</commit_message>
<xml_diff>
--- a/Tender_Summary.xlsx
+++ b/Tender_Summary.xlsx
@@ -39,7 +39,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -49,6 +49,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4E4"/>
       </patternFill>
     </fill>
   </fills>
@@ -78,12 +88,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -562,7 +578,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>GEM/2026/B/7920051 / NIT Ref NO: 9900330303 - Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+          <t>GEM/2026/B/7920051 - 103392745</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -572,74 +588,180 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
+          <t>Statutory audit of ash disposal</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>1 Month(s) (Audit report to be submitted before 31.08.2026)</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Rs. 145600.0</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Lumpsum basis (to be quoted by bidder in financial bid)</t>
+          <t>1 Month(s)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Rs. 145,600  [as written: 145600.0]</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>NOT FOUND - verify manually</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>- Minimum average annual turnover required: Rs. 51 Lakhs in preceding 3 financial years (2021-2022, 2020-2021, 2019-2020)
-- Only CPCB authorized Auditors shall undertake the compliance audit for ash disposal for NTPC Solapur as per MOEF&amp;CC notification dated 31.12.2021
-- Bidder must be a Class-I Local Supplier
-- Bidder should not be under any banning/suspension/withholding with NTPC Ltd.
-- Self-declarations required regarding insolvency, bankruptcy, liquidation, and absence of conflict of interest
-- Mandatory registrations: PAN, GSTIN</t>
+          <t>Eligibility Criteria
+Sub-Question
+Answer
+1. Minimum
+average annual
+turnover
+required:
+51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
+2. OEM turnover
+requirement:
+NA
+3. Financial
+years for
+Preceding three (3) financial years. The specific years are 2021-2022, 2020-
+2021, and 2019-2020.
+turnover
+consideration:
+4. Documents
+required to
+prove turnover:
+Audited financial statements for the last 3 financial years.
+If audited results for the last preceding financial year are not available,
+a certification of financial statement from a practicing chartered
+accountant.
+Certificate from the CEO/CFO of the Holding Company stating that the
+unaudited unconsolidated financial statements form part of the
+consolidated financial statements of the Holding Company, is enclosed
+as per the format at Appendix-A to Attachment 3A2.
+5. Experience
+required (years
+and type):
+The bidder must be a LOCAL SUPPLIER. Specific years of experience are
+not explicitly mentioned, but past experience related to the scope of work is
+required as per Attachment 3 and 4. For MSEs, the experience requirement is
+also subject to "Udyam Registration" and "Major Activity" not being
+"TRADING".
+6. Past
+performance /
+similar work
+experience:
+Details of past experience, such as authentic Work Orders/ Purchase
+Orders/ Letter of Awards/ Contract Agreements, and client certificates,
+completion certificate, etc., are required.
+Bidder is not permitted to quote more than 3 (three) times the reference
+documents like Work Orders/Purchase Orders/Letter of
+Awards/Contract Agreement, client certificates etc. for each Qualifying
+Requirement criteria.
+7. Exemptions
+from past
+performance
+requirements:
+NA
+8. Exemptions
+for MSE /
+MSME / Start-
+ups:
+MSEs registered with District Industries Centres or Khadi and Village
+Industries Commission or Khadi and Village Industries Board or Coir
+Board or National Small Industries Corporation or Directorate of
+Handicrafts and Handloom or any other body specified by Ministry o</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>- Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur
-- Verification of ash generation data based on coal receipt/consumption records and average ash content, comparing with annual compliance report
-- Verification of fly ash and bottom ash utilization data supplied to user agencies, comparing with annual compliance report
-- Verification of ash disposal into ash ponds (difference of ash generation and utilization)
-- Assessment of total ash storage in operational and un-operational ash ponds and available storage capacity
-- Assessment of ash slurry disposal and ash water re-circulation system (AWRS), water ratio, recycled water, and environmental discharge
-- Recommendations based on gap analysis for better improvement and statutory compliance
-- Final report submission in line with CPCB SOP before 31.08.2026</t>
+          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report
+to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the
+CPCB SOP/Guidelines etc in this regard.
+3
+Technical Requirement/Terms &amp; Conditions
+Audit shall be carried out as per the Ministry of Environment, Forest and Climate
+Change Notification, S.O. 5481(E), Dtd: 31st December 2021 and its subsequent
+amendments issued by ministry from time to time.
+The work involves the following:.
+i.
+Verification of ash generation data pertaining to the financial year based on
+inspection of records of coal receipt/consumption and average ash content
+in coal, and comparison of this data with the information provided by the
+power plant in the annual compliance report.
+ii.
+Verification of fly ash and bottom ash utilization data pertaining to the
+financial year based on inspection of records of ash supplied to the user
+agencies covered under permitted uses/avenues, and comparison of this
+data with the information provided by the power plant in the annual
+compliance report.
+iii.
+Verification of the ash disposal into ash ponds data pertaining to the
+financial year (i.e. difference of ash generation and ash utilization, as above),
+and comparison of this data with the information provided by the power
+plant in the annual compliance report.
+iv.
+Assessment of total ash storage in operational and un-operation ash ponds
+and available storage capacity for further disposal at the end of financial
+year based on details and drawings of ash ponds provided by the power
+plant and ground verification of the information provided, and comparison
+of the storage and storage capacity with the information provided by the
+power plant in the annual compliance report.
+v.
+Assessment of ash slurry disposal and ash water re-circulation system used
+during the financial year, in respect ratio of water in the ash disposed to ash
+ponds, water used for ash slurry disposal to ash ponds, ash water r</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Liquidated Damages (LD): Applicable; Rs. 5,000/- per day penalty on either party for failure to provide necessary information sought by Independent Engineer during investigation in a time bound manner</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Not Applicable</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>5.0% of the total Contract Price (2.5% of contract value for MSE-SC/ST and MSE-Women vendors)</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Not Applicable</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
+          <t>GCC clause-25.5.1
+As per GCC
+60. ITB Clause 4.0
+i. Bidder is advised to visit, inspect and examine the site(s) where the works are to
+be executed and its surroundings and obtain for itself on its own responsibility all
+information that may be necessary for preparing the bid and satisfy themselves
+before submitting their tenders as to the nature of the ground and sub-soil (so far
+as is practicable), the form and nature of the site, the means of access to the site,
+the accommodation they may require and in general, shall themselves obtain all
+necessary information as to risks, contingencies and other circumstances which
+may influence or effect their tender.
+A Bidder shall be deemed to have full knowledge of the site, whether he inspects
+it or not and no extra charges consequent on any misunderstanding or otherwise
+shall be allowed. The costs of visiting the site shall be borne by the bidder fully.
+61.
+ii. Local Conditions:
+a) It will be imperative on each Bidder to fully inform himself of all local
+conditions and factors which may have any effect on the execution of the
+works covered under these documents &amp; specifications and to take the same
+into account while submitting his bid.
+b) Successful bidder shall make all effort and cooperate with the EIC in
+maintaining cordial, harmonious and conducive environment and industrial
+relations with respect to and connected to this work, so that smooth and
+effective execution of the work is achieved.
+c) Keeping the above in view, the bidder shall do required liasoning with local</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Not Applicable / Nil (as stated)</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>5.0% of the total Contract Price</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Not Applicable / Nil (as stated)</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>25-08-2026 11:00:00</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>clean</t>
+          <t>6 field(s): Tender Estimated Cost, Assignment Fees, Tender EMD, Tender SD, Tender Fees, Tender Submission Date</t>
         </is>
       </c>
     </row>
@@ -669,42 +791,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Tender</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Final Value</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Source (file, page)</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Rules layer read</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>AI layer read</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Flag</t>
         </is>
@@ -723,7 +845,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>GEM/2026/B/7920051 / NIT Ref NO: 9900330303 - Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+          <t>GEM/2026/B/7920051 - 103392745</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -741,11 +863,7 @@
           <t>GEM/2026/B/7920051 - 103392745</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>GEM/2026/B/7920051 / NIT Ref NO: 9900330303 - Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
-        </is>
-      </c>
+      <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="42" customHeight="1">
@@ -779,11 +897,7 @@
           <t>1045-Solapur STPP, Solapur STPP, AT-FATATEWADI, PO-HOTGI STATION, SOUTH SOLAPUR, SOLAPUR, Maharashtra-413215</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>1045-Solapur STPP, Solapur STPP, AT-FATATEWADI, PO-HOTGI STATION, SOUTH SOLAPUR, SOLAPUR, Maharashtra-413215</t>
-        </is>
-      </c>
+      <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="42" customHeight="1">
@@ -799,12 +913,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
+          <t>Statutory audit of ash disposal</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>210347180.pdf (p.2)</t>
+          <t>Tender-Summary-103392745.pdf (p.1)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -817,11 +931,7 @@
           <t>Statutory audit of ash disposal</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
-        </is>
-      </c>
+      <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="42" customHeight="1">
@@ -837,12 +947,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>1 Month(s) (Audit report to be submitted before 31.08.2026)</t>
+          <t>1 Month(s)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>210347180.pdf (p.5)</t>
+          <t>Tender-Summary-103392745.pdf (p.1)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -855,84 +965,72 @@
           <t>1 Month(s)</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>1 Month(s) (Audit report to be submitted before 31.08.2026)</t>
-        </is>
-      </c>
+      <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>5. Tender Estimated Cost</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Rs. 145600.0</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Rs. 145,600  [as written: 145600.0]</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Tender-Summary-103392745.pdf (p.2)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Rs. 145,600  [as written: 145600.0]</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Rs. 145600.0</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>single reader - AI cross-check did not run</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>6. Assignment Fees</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Lumpsum basis (to be quoted by bidder in financial bid)</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>210347184.pdf (p.10)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Lumpsum basis (to be quoted by bidder in financial bid)</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>NOT FOUND - verify manually</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -946,26 +1044,6 @@
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>- Minimum average annual turnover required: Rs. 51 Lakhs in preceding 3 financial years (2021-2022, 2020-2021, 2019-2020)
-- Only CPCB authorized Auditors shall undertake the compliance audit for ash disposal for NTPC Solapur as per MOEF&amp;CC notification dated 31.12.2021
-- Bidder must be a Class-I Local Supplier
-- Bidder should not be under any banning/suspension/withholding with NTPC Ltd.
-- Self-declarations required regarding insolvency, bankruptcy, liquidation, and absence of conflict of interest
-- Mandatory registrations: PAN, GSTIN</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Tender-Summary-103392745.pdf (p.3)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Eligibility Criteria
 Sub-Question
@@ -1014,16 +1092,66 @@
 documents li</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>- Minimum average annual turnover required: Rs. 51 Lakhs in preceding 3 financial years (2021-2022, 2020-2021, 2019-2020)
-- Only CPCB authorized Auditors shall undertake the compliance audit for ash disposal for NTPC Solapur as per MOEF&amp;CC notification dated 31.12.2021
-- Bidder must be a Class-I Local Supplier
-- Bidder should not be under any banning/suspension/withholding with NTPC Ltd.
-- Self-declarations required regarding insolvency, bankruptcy, liquidation, and absence of conflict of interest
-- Mandatory registrations: PAN, GSTIN</t>
-        </is>
-      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Tender-Summary-103392745.pdf (p.3)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Eligibility Criteria
+Sub-Question
+Answer
+1. Minimum
+average annual
+turnover
+required:
+51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
+2. OEM turnover
+requirement:
+NA
+3. Financial
+years for
+Preceding three (3) financial years. The specific years are 2021-2022, 2020-
+2021, and 2019-2020.
+turnover
+consideration:
+4. Documents
+required to
+prove turnover:
+Audited financial statements for the last 3 financial years.
+If audited results for the last preceding financial year are not available,
+a certification of financial statement from a practicing chartered
+accountant.
+Certificate from the CEO/CFO of the Holding Company stating that the
+unaudited unconsolidated financial statements form part of the
+consolidated financial statements of the Holding Company, is enclosed
+as per the format at Appendix-A to Attachment 3A2.
+5. Experience
+required (years
+and type):
+The bidder must be a LOCAL SUPPLIER. Specific years of experience are
+not explicitly mentioned, but past experience related to the scope of work is
+required as per Attachment 3 and 4. For MSEs, the experience requirement is
+also subject to "Udyam Registration" and "Major Activity" not being
+"TRADING".
+6. Past
+performance /
+similar work
+experience:
+Details of past experience, such as authentic Work Orders/ Purchase
+Orders/ Letter of Awards/ Contract Agreements, and client certificates,
+completion certificate, etc., are required.
+Bidder is not permitted to quote more than 3 (three) times the reference
+documents li</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="42" customHeight="1">
@@ -1038,28 +1166,6 @@
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>- Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur
-- Verification of ash generation data based on coal receipt/consumption records and average ash content, comparing with annual compliance report
-- Verification of fly ash and bottom ash utilization data supplied to user agencies, comparing with annual compliance report
-- Verification of ash disposal into ash ponds (difference of ash generation and utilization)
-- Assessment of total ash storage in operational and un-operational ash ponds and available storage capacity
-- Assessment of ash slurry disposal and ash water re-circulation system (AWRS), water ratio, recycled water, and environmental discharge
-- Recommendations based on gap analysis for better improvement and statutory compliance
-- Final report submission in line with CPCB SOP before 31.08.2026</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>210347180.pdf (p.3)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report
 to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the
@@ -1091,18 +1197,49 @@
 and available storage capacity for further disposal at the end o</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>- Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur
-- Verification of ash generation data based on coal receipt/consumption records and average ash content, comparing with annual compliance report
-- Verification of fly ash and bottom ash utilization data supplied to user agencies, comparing with annual compliance report
-- Verification of ash disposal into ash ponds (difference of ash generation and utilization)
-- Assessment of total ash storage in operational and un-operational ash ponds and available storage capacity
-- Assessment of ash slurry disposal and ash water re-circulation system (AWRS), water ratio, recycled water, and environmental discharge
-- Recommendations based on gap analysis for better improvement and statutory compliance
-- Final report submission in line with CPCB SOP before 31.08.2026</t>
-        </is>
-      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>210347180.pdf (p.3)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report
+to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the
+CPCB SOP/Guidelines etc in this regard.
+3
+Technical Requirement/Terms &amp; Conditions
+Audit shall be carried out as per the Ministry of Environment, Forest and Climate
+Change Notification, S.O. 5481(E), Dtd: 31st December 2021 and its subsequent
+amendments issued by ministry from time to time.
+The work involves the following:.
+i.
+Verification of ash generation data pertaining to the financial year based on
+inspection of records of coal receipt/consumption and average ash content
+in coal, and comparison of this data with the information provided by the
+power plant in the annual compliance report.
+ii.
+Verification of fly ash and bottom ash utilization data pertaining to the
+financial year based on inspection of records of ash supplied to the user
+agencies covered under permitted uses/avenues, and comparison of this
+data with the information provided by the power plant in the annual
+compliance report.
+iii.
+Verification of the ash disposal into ash ponds data pertaining to the
+financial year (i.e. difference of ash generation and ash utilization, as above),
+and comparison of this data with the information provided by the power
+plant in the annual compliance report.
+iv.
+Assessment of total ash storage in operational and un-operation ash ponds
+and available storage capacity for further disposal at the end o</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
     </row>
     <row r="10" ht="42" customHeight="1">
@@ -1117,21 +1254,6 @@
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Liquidated Damages (LD): Applicable; Rs. 5,000/- per day penalty on either party for failure to provide necessary information sought by Independent Engineer during investigation in a time bound manner</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>210347180.pdf (p.5)</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>GCC clause-25.5.1
 As per GCC
@@ -1160,164 +1282,199 @@
 c) Keeping the above in view, the</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Liquidated Damages (LD): Applicable; Rs. 5,000/- per day penalty on either party for failure to provide necessary information sought by Independent Engineer during investigation in a time bound manner</t>
-        </is>
-      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>210347184.pdf (p.22)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>GCC clause-25.5.1
+As per GCC
+60. ITB Clause 4.0
+i. Bidder is advised to visit, inspect and examine the site(s) where the works are to
+be executed and its surroundings and obtain for itself on its own responsibility all
+information that may be necessary for preparing the bid and satisfy themselves
+before submitting their tenders as to the nature of the ground and sub-soil (so far
+as is practicable), the form and nature of the site, the means of access to the site,
+the accommodation they may require and in general, shall themselves obtain all
+necessary information as to risks, contingencies and other circumstances which
+may influence or effect their tender.
+A Bidder shall be deemed to have full knowledge of the site, whether he inspects
+it or not and no extra charges consequent on any misunderstanding or otherwise
+shall be allowed. The costs of visiting the site shall be borne by the bidder fully.
+61.
+ii. Local Conditions:
+a) It will be imperative on each Bidder to fully inform himself of all local
+conditions and factors which may have any effect on the execution of the
+works covered under these documents &amp; specifications and to take the same
+into account while submitting his bid.
+b) Successful bidder shall make all effort and cooperate with the EIC in
+maintaining cordial, harmonious and conducive environment and industrial
+relations with respect to and connected to this work, so that smooth and
+effective execution of the work is achieved.
+c) Keeping the above in view, the</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>10. Tender EMD</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Not Applicable</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Not Applicable / Nil (as stated)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Tender-Summary-103392745.pdf (p.2)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Not Applicable / Nil (as stated)</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Not Applicable</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>single reader - AI cross-check did not run</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>11. Tender SD</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>5.0% of the total Contract Price (2.5% of contract value for MSE-SC/ST and MSE-Women vendors)</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>5.0% of the total Contract Price</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>210347184.pdf (p.17)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>5.0% of the total Contract Price</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>5.0% of the total Contract Price (2.5% of contract value for MSE-SC/ST and MSE-Women vendors)</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>single reader - AI cross-check did not run</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>12. Tender Fees</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Not Applicable</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Not Applicable / Nil (as stated)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>210347179.pdf (p.3)</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Not Applicable / Nil (as stated)</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Not Applicable</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>single reader - AI cross-check did not run</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>13. Tender Submission Date</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>25-08-2026 11:00:00</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Tender-Summary-103392745.pdf (p.1)</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>25-08-2026 11:00:00</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>25-08-2026 11:00:00</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>single reader - AI cross-check did not run</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1341,259 +1498,259 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Tender</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Pages read</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Pages needing OCR</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>210347177.pdf</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="4" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>210347178.pdf</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="4" t="inlineStr"/>
+      <c r="E3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>210347179.pdf</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="4" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>210347180.pdf</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="4" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>210347181.pdf</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="4" t="inlineStr"/>
+      <c r="E6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>210347182.pdf</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="4" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>210347183.pdf</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="4" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>210347184.pdf</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="4" t="inlineStr"/>
+      <c r="E9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>ATTACHMENT - 9 (2).pdf</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="4" t="inlineStr"/>
+      <c r="E10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>ATTACHMENT - 9.pdf</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="4" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Tender-Summary-103392745.pdf</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="4" t="inlineStr"/>
+      <c r="E12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>TENDER.pdf</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="6" t="n">
         <v>417</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="4" t="inlineStr"/>
+      <c r="E13" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1614,132 +1771,132 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>How to read this workbook</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr"/>
+      <c r="B1" s="8" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Tender Summary</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>One row per tender folder, the 13 requested fields.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>For every field: the source file and page it came from, plus what each of the two independent readers (rules and AI) read. Use this to verify a value in seconds.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Documents Read</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Which files were opened, how many pages, how many needed OCR.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr"/>
-      <c r="B5" s="6" t="inlineStr"/>
+      <c r="A5" s="7" t="inlineStr"/>
+      <c r="B5" s="8" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Cell colours</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
+      <c r="B6" s="8" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Amber</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Needs your eye: the two readers disagreed, confidence was low, or the value came off a scanned page via OCR.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Not stated anywhere in the documents that were read.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr"/>
-      <c r="B9" s="6" t="inlineStr"/>
+      <c r="A9" s="7" t="inlineStr"/>
+      <c r="B9" s="8" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Important</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>This tool eliminates the typing, not the review. Always confirm EMD, fees, and the submission deadline against the source page before acting on them.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Single reader</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Without a Gemini API key only the rules layer runs. Money and date fields are then capped at medium confidence and flagged, because nothing cross-checked them.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Percentages</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Security deposit and performance guarantees are normally a percentage of contract value, so that is what is reported. A rupee figure sitting next to a phrase like "up to" is a threshold, not the amount payable, and is flagged as such.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Excluded</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>WORKING FOLDER is skipped by design - it holds your own draft submissions, not the department's tender documents.</t>
         </is>

</xml_diff>

<commit_message>
Fix NOT FOUND override bug and max chunks truncation
</commit_message>
<xml_diff>
--- a/Tender_Summary.xlsx
+++ b/Tender_Summary.xlsx
@@ -39,7 +39,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -49,11 +49,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -88,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -97,9 +92,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -578,7 +570,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>GEM/2026/B/7920051 - 103392745</t>
+          <t>Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -588,180 +580,66 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal</t>
+          <t>Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>1 Month(s)</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Rs. 145,600  [as written: 145600.0]</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Rs. 145,600</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>NOT FOUND - verify manually</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Eligibility Criteria
-Sub-Question
-Answer
-1. Minimum
-average annual
-turnover
-required:
-51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
-2. OEM turnover
-requirement:
-NA
-3. Financial
-years for
-Preceding three (3) financial years. The specific years are 2021-2022, 2020-
-2021, and 2019-2020.
-turnover
-consideration:
-4. Documents
-required to
-prove turnover:
-Audited financial statements for the last 3 financial years.
-If audited results for the last preceding financial year are not available,
-a certification of financial statement from a practicing chartered
-accountant.
-Certificate from the CEO/CFO of the Holding Company stating that the
-unaudited unconsolidated financial statements form part of the
-consolidated financial statements of the Holding Company, is enclosed
-as per the format at Appendix-A to Attachment 3A2.
-5. Experience
-required (years
-and type):
-The bidder must be a LOCAL SUPPLIER. Specific years of experience are
-not explicitly mentioned, but past experience related to the scope of work is
-required as per Attachment 3 and 4. For MSEs, the experience requirement is
-also subject to "Udyam Registration" and "Major Activity" not being
-"TRADING".
-6. Past
-performance /
-similar work
-experience:
-Details of past experience, such as authentic Work Orders/ Purchase
-Orders/ Letter of Awards/ Contract Agreements, and client certificates,
-completion certificate, etc., are required.
-Bidder is not permitted to quote more than 3 (three) times the reference
-documents like Work Orders/Purchase Orders/Letter of
-Awards/Contract Agreement, client certificates etc. for each Qualifying
-Requirement criteria.
-7. Exemptions
-from past
-performance
-requirements:
-NA
-8. Exemptions
-for MSE /
-MSME / Start-
-ups:
-MSEs registered with District Industries Centres or Khadi and Village
-Industries Commission or Khadi and Village Industries Board or Coir
-Board or National Small Industries Corporation or Directorate of
-Handicrafts and Handloom or any other body specified by Ministry o</t>
+          <t>1. Only CPCB authorized Auditors shall undertake the compliance audit for ash disposal for NTPC Solapur as per MOEF&amp;CC notification dated 31.12.2021 and its subsequent amendments. (Bidder to submit documentary evidence in this regard, in absence of same Bids shall be liable for rejection.)
+2. The bidder should not be under any banning/suspension/withholding with NTPC Ltd.
+3. All the bidders have to submit the GTE template PAN, GSTIN and enlistment certificate issued OR copy of the email for this package sent by the buyer/tender inviting authority.
+4. MSE Purchase Preference: Purchase preference will be given to MSEs having valid Udyam Certificate and whose credentials are validated online through Udyam Registration portal. If L-1 is not an MSE and MSE Seller(s) has/have quoted price within L-1+ 15% of margin of purchase preference, such MSE Seller shall be given opportunity to match L-1 price and contract will be awarded for 100% of total value.
+5. EMD exemption for: IIMs/IITs/ NITs/ IISc./ CBRI/ CPRI/ GSI/CWPRS/ CWC/ NEERI/ CSIR Labs and other Govt. Institutes/agencies (excluding PSUs).</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report
-to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the
-CPCB SOP/Guidelines etc in this regard.
-3
-Technical Requirement/Terms &amp; Conditions
-Audit shall be carried out as per the Ministry of Environment, Forest and Climate
-Change Notification, S.O. 5481(E), Dtd: 31st December 2021 and its subsequent
-amendments issued by ministry from time to time.
-The work involves the following:.
-i.
-Verification of ash generation data pertaining to the financial year based on
-inspection of records of coal receipt/consumption and average ash content
-in coal, and comparison of this data with the information provided by the
-power plant in the annual compliance report.
-ii.
-Verification of fly ash and bottom ash utilization data pertaining to the
-financial year based on inspection of records of ash supplied to the user
-agencies covered under permitted uses/avenues, and comparison of this
-data with the information provided by the power plant in the annual
-compliance report.
-iii.
-Verification of the ash disposal into ash ponds data pertaining to the
-financial year (i.e. difference of ash generation and ash utilization, as above),
-and comparison of this data with the information provided by the power
-plant in the annual compliance report.
-iv.
-Assessment of total ash storage in operational and un-operation ash ponds
-and available storage capacity for further disposal at the end of financial
-year based on details and drawings of ash ponds provided by the power
-plant and ground verification of the information provided, and comparison
-of the storage and storage capacity with the information provided by the
-power plant in the annual compliance report.
-v.
-Assessment of ash slurry disposal and ash water re-circulation system used
-during the financial year, in respect ratio of water in the ash disposed to ash
-ponds, water used for ash slurry disposal to ash ponds, ash water r</t>
+          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under permitted uses/avenues, and comparison of this data with the information provided by the power plant in the annual compliance report. iii. Verification of the ash disposal into ash ponds data pertaining to the financial year (i.e. difference of ash generation and ash utilization, as above), and comparison of this data with the information provided by the power plant in the annual compliance report. iv. Assessment of total ash storage in operational and un-operation ash ponds and available storage capacity for further disposal at the end of financial year based on details and drawings of ash ponds provided by the power plant and ground verification of the information provided, and comparison of the storage and storage capacity with the information provided by the power plant in the annual compliance report. v. Assessment of ash slurry disposal and ash water re-circulation system used during the financial year, in respect ratio of water in the ash disposed to ash ponds, water used for ash slurry disposal to ash ponds, ash water recycled through AWRS, and ash water discharged into environment based on inspection of records provided by the power plant and ground verification, including the condition of surrounding environment in respect of ash released or breached, and comparison of the ground situat</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>GCC clause-25.5.1
-As per GCC
-60. ITB Clause 4.0
-i. Bidder is advised to visit, inspect and examine the site(s) where the works are to
-be executed and its surroundings and obtain for itself on its own responsibility all
-information that may be necessary for preparing the bid and satisfy themselves
-before submitting their tenders as to the nature of the ground and sub-soil (so far
-as is practicable), the form and nature of the site, the means of access to the site,
-the accommodation they may require and in general, shall themselves obtain all
-necessary information as to risks, contingencies and other circumstances which
-may influence or effect their tender.
-A Bidder shall be deemed to have full knowledge of the site, whether he inspects
-it or not and no extra charges consequent on any misunderstanding or otherwise
-shall be allowed. The costs of visiting the site shall be borne by the bidder fully.
-61.
-ii. Local Conditions:
-a) It will be imperative on each Bidder to fully inform himself of all local
-conditions and factors which may have any effect on the execution of the
-works covered under these documents &amp; specifications and to take the same
-into account while submitting his bid.
-b) Successful bidder shall make all effort and cooperate with the EIC in
-maintaining cordial, harmonious and conducive environment and industrial
-relations with respect to and connected to this work, so that smooth and
-effective execution of the work is achieved.
-c) Keeping the above in view, the bidder shall do required liasoning with local</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>Not Applicable / Nil (as stated)</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>5.0% of the total Contract Price</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>Not Applicable / Nil (as stated)</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
+          <t>LD: Applicable</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>25-08-2026 11:00:00</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>6 field(s): Tender Estimated Cost, Assignment Fees, Tender EMD, Tender SD, Tender Fees, Tender Submission Date</t>
+          <t>1 field(s): Assignment Fees</t>
         </is>
       </c>
     </row>
@@ -791,42 +669,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Tender</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Final Value</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Source (file, page)</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Rules layer read</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>AI layer read</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Flag</t>
         </is>
@@ -845,25 +723,29 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Tender-Summary-103392745.pdf (p.1)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>GEM/2026/B/7920051 - 103392745</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Tender-Summary-103392745.pdf (p.1)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>GEM/2026/B/7920051 - 103392745</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="42" customHeight="1">
@@ -897,7 +779,11 @@
           <t>1045-Solapur STPP, Solapur STPP, AT-FATATEWADI, PO-HOTGI STATION, SOUTH SOLAPUR, SOLAPUR, Maharashtra-413215</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>1045-Solapur STPP, Solapur STPP, AT-FATATEWADI, PO-HOTGI STATION, SOUTH SOLAPUR, SOLAPUR, Maharashtra-413215</t>
+        </is>
+      </c>
       <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="42" customHeight="1">
@@ -913,25 +799,29 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>210347180.pdf (p.2)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>Statutory audit of ash disposal</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Tender-Summary-103392745.pdf (p.1)</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Statutory audit of ash disposal</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="42" customHeight="1">
@@ -947,86 +837,90 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Tender-Summary-103392745.pdf (p.1)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>1 Month(s)</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Tender-Summary-103392745.pdf (p.1)</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>5. Tender Estimated Cost</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Rs. 145,600</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Tender-Summary-103392745.pdf (p.2)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>1 Month(s)</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>5. Tender Estimated Cost</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Rs. 145,600  [as written: 145600.0]</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Tender-Summary-103392745.pdf (p.2)</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Rs. 145,600  [as written: 145600.0]</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>single reader - AI cross-check did not run</t>
-        </is>
-      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Rs. 145,600</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>6. Assignment Fees</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>NOT FOUND - verify manually</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
@@ -1044,6 +938,25 @@
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>1. Only CPCB authorized Auditors shall undertake the compliance audit for ash disposal for NTPC Solapur as per MOEF&amp;CC notification dated 31.12.2021 and its subsequent amendments. (Bidder to submit documentary evidence in this regard, in absence of same Bids shall be liable for rejection.)
+2. The bidder should not be under any banning/suspension/withholding with NTPC Ltd.
+3. All the bidders have to submit the GTE template PAN, GSTIN and enlistment certificate issued OR copy of the email for this package sent by the buyer/tender inviting authority.
+4. MSE Purchase Preference: Purchase preference will be given to MSEs having valid Udyam Certificate and whose credentials are validated online through Udyam Registration portal. If L-1 is not an MSE and MSE Seller(s) has/have quoted price within L-1+ 15% of margin of purchase preference, such MSE Seller shall be given opportunity to match L-1 price and contract will be awarded for 100% of total value.
+5. EMD exemption for: IIMs/IITs/ NITs/ IISc./ CBRI/ CPRI/ GSI/CWPRS/ CWC/ NEERI/ CSIR Labs and other Govt. Institutes/agencies (excluding PSUs).</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>210347177.pdf (p.5)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Eligibility Criteria
 Sub-Question
@@ -1092,66 +1005,15 @@
 documents li</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Tender-Summary-103392745.pdf (p.3)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Eligibility Criteria
-Sub-Question
-Answer
-1. Minimum
-average annual
-turnover
-required:
-51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
-2. OEM turnover
-requirement:
-NA
-3. Financial
-years for
-Preceding three (3) financial years. The specific years are 2021-2022, 2020-
-2021, and 2019-2020.
-turnover
-consideration:
-4. Documents
-required to
-prove turnover:
-Audited financial statements for the last 3 financial years.
-If audited results for the last preceding financial year are not available,
-a certification of financial statement from a practicing chartered
-accountant.
-Certificate from the CEO/CFO of the Holding Company stating that the
-unaudited unconsolidated financial statements form part of the
-consolidated financial statements of the Holding Company, is enclosed
-as per the format at Appendix-A to Attachment 3A2.
-5. Experience
-required (years
-and type):
-The bidder must be a LOCAL SUPPLIER. Specific years of experience are
-not explicitly mentioned, but past experience related to the scope of work is
-required as per Attachment 3 and 4. For MSEs, the experience requirement is
-also subject to "Udyam Registration" and "Major Activity" not being
-"TRADING".
-6. Past
-performance /
-similar work
-experience:
-Details of past experience, such as authentic Work Orders/ Purchase
-Orders/ Letter of Awards/ Contract Agreements, and client certificates,
-completion certificate, etc., are required.
-Bidder is not permitted to quote more than 3 (three) times the reference
-documents li</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>1. Only CPCB authorized Auditors shall undertake the compliance audit for ash disposal for NTPC Solapur as per MOEF&amp;CC notification dated 31.12.2021 and its subsequent amendments. (Bidder to submit documentary evidence in this regard, in absence of same Bids shall be liable for rejection.)
+2. The bidder should not be under any banning/suspension/withholding with NTPC Ltd.
+3. All the bidders have to submit the GTE template PAN, GSTIN and enlistment certificate issued OR copy of the email for this package sent by the buyer/tender inviting authority.
+4. MSE Purchase Preference: Purchase preference will be given to MSEs having valid Udyam Certificate and whose credentials are validated online through Udyam Registration portal. If L-1 is not an MSE and MSE Seller(s) has/have quoted price within L-1+ 15% of margin of purchase preference, such MSE Seller shall be given opportunity to match L-1 price and contract will be awarded for 100% of total value.
+5. EMD exemption for: IIMs/IITs/ NITs/ IISc./ CBRI/ CPRI/ GSI/CWPRS/ CWC/ NEERI/ CSIR Labs and other Govt. Institutes/agencies (excluding PSUs).</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="42" customHeight="1">
@@ -1166,6 +1028,21 @@
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under permitted uses/avenues, and comparison of this data with the information provided by the power plant in the annual compliance report. iii. Verification of the ash disposal into ash ponds data pertaining to the financial year (i.e. difference of ash generation and ash utilization, as above), and comparison of this data with the information provided by the power plant in the annual compliance report. iv. Assessment of total ash storage in operational and un-operation ash ponds and available storage capacity for further disposal at the end of financial year based on details and drawings of ash ponds provided by the power plant and ground verification of the information provided, and comparison of the storage and storage capacity with the information provided by the power plant in the annual compliance report.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>210347180.pdf (p.3)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report
 to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the
@@ -1197,49 +1074,11 @@
 and available storage capacity for further disposal at the end o</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>210347180.pdf (p.3)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report
-to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the
-CPCB SOP/Guidelines etc in this regard.
-3
-Technical Requirement/Terms &amp; Conditions
-Audit shall be carried out as per the Ministry of Environment, Forest and Climate
-Change Notification, S.O. 5481(E), Dtd: 31st December 2021 and its subsequent
-amendments issued by ministry from time to time.
-The work involves the following:.
-i.
-Verification of ash generation data pertaining to the financial year based on
-inspection of records of coal receipt/consumption and average ash content
-in coal, and comparison of this data with the information provided by the
-power plant in the annual compliance report.
-ii.
-Verification of fly ash and bottom ash utilization data pertaining to the
-financial year based on inspection of records of ash supplied to the user
-agencies covered under permitted uses/avenues, and comparison of this
-data with the information provided by the power plant in the annual
-compliance report.
-iii.
-Verification of the ash disposal into ash ponds data pertaining to the
-financial year (i.e. difference of ash generation and ash utilization, as above),
-and comparison of this data with the information provided by the power
-plant in the annual compliance report.
-iv.
-Assessment of total ash storage in operational and un-operation ash ponds
-and available storage capacity for further disposal at the end o</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under permitted uses/avenues, and comparison of this data with the information provided by the power plant in the annual compliance report. iii. Verification of the ash disposal into ash ponds data pertaining to the financial year (i.e. difference of ash generation and ash utilization, as above), and comparison of this data with the information provided by the power plant in the annual compliance report. iv. Assessment of total ash storage in operational and un-operation ash ponds and available storage capacity for further disposal at the end of financial year based on details and drawings of ash ponds provided by the power plant and ground verification of the information provided, and comparison of the storage and storage capacity with the information provided by the power plant in the annual compliance report.</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr"/>
     </row>
     <row r="10" ht="42" customHeight="1">
@@ -1254,6 +1093,21 @@
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>LD: Applicable</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>210347180.pdf (p.5)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>GCC clause-25.5.1
 As per GCC
@@ -1282,199 +1136,164 @@
 c) Keeping the above in view, the</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>210347184.pdf (p.22)</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>LD: Applicable</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>10. Tender EMD</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>210347177.pdf (p.2)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>GCC clause-25.5.1
-As per GCC
-60. ITB Clause 4.0
-i. Bidder is advised to visit, inspect and examine the site(s) where the works are to
-be executed and its surroundings and obtain for itself on its own responsibility all
-information that may be necessary for preparing the bid and satisfy themselves
-before submitting their tenders as to the nature of the ground and sub-soil (so far
-as is practicable), the form and nature of the site, the means of access to the site,
-the accommodation they may require and in general, shall themselves obtain all
-necessary information as to risks, contingencies and other circumstances which
-may influence or effect their tender.
-A Bidder shall be deemed to have full knowledge of the site, whether he inspects
-it or not and no extra charges consequent on any misunderstanding or otherwise
-shall be allowed. The costs of visiting the site shall be borne by the bidder fully.
-61.
-ii. Local Conditions:
-a) It will be imperative on each Bidder to fully inform himself of all local
-conditions and factors which may have any effect on the execution of the
-works covered under these documents &amp; specifications and to take the same
-into account while submitting his bid.
-b) Successful bidder shall make all effort and cooperate with the EIC in
-maintaining cordial, harmonious and conducive environment and industrial
-relations with respect to and connected to this work, so that smooth and
-effective execution of the work is achieved.
-c) Keeping the above in view, the</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>10. Tender EMD</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Not Applicable / Nil (as stated)</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Tender-Summary-103392745.pdf (p.2)</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>11. Tender SD</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>210347180.pdf (p.5)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>5.0% of the total Contract Price</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>12. Tender Fees</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>210347179.pdf (p.3)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Not Applicable / Nil (as stated)</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>single reader - AI cross-check did not run</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>11. Tender SD</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>5.0% of the total Contract Price</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>210347184.pdf (p.17)</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>5.0% of the total Contract Price</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>single reader - AI cross-check did not run</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>12. Tender Fees</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Not Applicable / Nil (as stated)</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>210347179.pdf (p.3)</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Not Applicable / Nil (as stated)</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>single reader - AI cross-check did not run</t>
-        </is>
-      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
     </row>
     <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>13. Tender Submission Date</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>25-08-2026 11:00:00</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Tender-Summary-103392745.pdf (p.1)</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>210347177.pdf (p.1)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>25-08-2026 11:00:00</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>single reader - AI cross-check did not run</t>
-        </is>
-      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>25-08-2026 11:00:00</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1498,259 +1317,259 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Tender</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Pages read</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Pages needing OCR</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>210347177.pdf</t>
         </is>
       </c>
-      <c r="C2" s="6" t="n">
+      <c r="C2" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="D2" s="6" t="n">
+      <c r="D2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="6" t="inlineStr"/>
+      <c r="E2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>210347178.pdf</t>
         </is>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="C3" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="6" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>210347179.pdf</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n">
+      <c r="C4" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="6" t="n">
+      <c r="D4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="6" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>210347180.pdf</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="6" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>210347181.pdf</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="6" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>210347182.pdf</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="6" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>210347183.pdf</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="6" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>210347184.pdf</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="6" t="inlineStr"/>
+      <c r="E9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>ATTACHMENT - 9 (2).pdf</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="6" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>ATTACHMENT - 9.pdf</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="D11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="6" t="inlineStr"/>
+      <c r="E11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Tender-Summary-103392745.pdf</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="6" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>TENDER.pdf</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="5" t="n">
         <v>417</v>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="6" t="inlineStr"/>
+      <c r="E13" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1771,132 +1590,132 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>How to read this workbook</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr"/>
+      <c r="B1" s="7" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Tender Summary</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>One row per tender folder, the 13 requested fields.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>For every field: the source file and page it came from, plus what each of the two independent readers (rules and AI) read. Use this to verify a value in seconds.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Documents Read</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Which files were opened, how many pages, how many needed OCR.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr"/>
-      <c r="B5" s="8" t="inlineStr"/>
+      <c r="A5" s="6" t="inlineStr"/>
+      <c r="B5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Cell colours</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr"/>
+      <c r="B6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Amber</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Needs your eye: the two readers disagreed, confidence was low, or the value came off a scanned page via OCR.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Not stated anywhere in the documents that were read.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr"/>
-      <c r="B9" s="8" t="inlineStr"/>
+      <c r="A9" s="6" t="inlineStr"/>
+      <c r="B9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Important</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>This tool eliminates the typing, not the review. Always confirm EMD, fees, and the submission deadline against the source page before acting on them.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Single reader</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Without a Gemini API key only the rules layer runs. Money and date fields are then capped at medium confidence and flagged, because nothing cross-checked them.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Percentages</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Security deposit and performance guarantees are normally a percentage of contract value, so that is what is reported. A rupee figure sitting next to a phrase like "up to" is a threshold, not the amount payable, and is flagged as such.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Excluded</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>WORKING FOLDER is skipped by design - it holds your own draft submissions, not the department's tender documents.</t>
         </is>

</xml_diff>

<commit_message>
Fix prose field merging to concatenate rather than overwrite
</commit_message>
<xml_diff>
--- a/Tender_Summary.xlsx
+++ b/Tender_Summary.xlsx
@@ -39,7 +39,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -49,11 +49,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4E4"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,15 +78,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -570,7 +562,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+          <t>Tender Id 103392745 - Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -593,18 +585,23 @@
           <t>Rs. 145,600</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND - verify manually</t>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>1. Only CPCB authorized Auditors shall undertake the compliance audit for ash disposal for NTPC Solapur as per MOEF&amp;CC notification dated 31.12.2021 and its subsequent amendments. (Bidder to submit documentary evidence in this regard, in absence of same Bids shall be liable for rejection.)
-2. The bidder should not be under any banning/suspension/withholding with NTPC Ltd.
-3. All the bidders have to submit the GTE template PAN, GSTIN and enlistment certificate issued OR copy of the email for this package sent by the buyer/tender inviting authority.
-4. MSE Purchase Preference: Purchase preference will be given to MSEs having valid Udyam Certificate and whose credentials are validated online through Udyam Registration portal. If L-1 is not an MSE and MSE Seller(s) has/have quoted price within L-1+ 15% of margin of purchase preference, such MSE Seller shall be given opportunity to match L-1 price and contract will be awarded for 100% of total value.
-5. EMD exemption for: IIMs/IITs/ NITs/ IISc./ CBRI/ CPRI/ GSI/CWPRS/ CWC/ NEERI/ CSIR Labs and other Govt. Institutes/agencies (excluding PSUs).</t>
+          <t>1. Minimum average annual turnover required: 51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
+2. OEM turnover requirement: NA.
+3. Financial years for preceding three (3) financial years: 2021-2022, 2020-2021, and 2019-2020.
+4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, as per Appendix-A to Attachment 3A2.
+5. Experience required (years and type): The bidder must be a LOCAL SUPPLIER. Specific years of experience are not explicitly mentioned, but past experience related to the scope of work is required as per Attachment 3 and 4. For MSEs, the experience requirement is also subject to "Udyam Registration" and "Major Activity" not being "TRADING".
+6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents for each Qualifying Requirement criteria.
+7. Exemptions from past performance requirements: NA.
+8. Exemptions for MSE / MSME / Start-ups: MSEs registered with appropriate bodies having UDYAM Registration for goods produced and services rendered are exempted from paying Earnest Money Deposit and are issued bid documents free of cost. MSE benefits are applicable for Service Contracts only, not for Works Contracts. Specific preference hierarchy for price band of L1 + 15% is outlined.
+9. Production capacity requirements: NA.
+10. Make in India requirements or preferences: Not Applicable. However, Class‑I local sup</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -614,12 +611,15 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>LD: Applicable</t>
+          <t>1. If a bidder after having been issued the Notification of Award, either does not sign the Contract Agreement or does not submit an acceptable Performance Security, resulting in retendering, the bidder shall be treated ineligible for participation in re-tendering of this particular package and dealt as per the provisions of policy for Debarment from Business Dealings.
+2. If a bidder after opening of the tender withdraws its offer within the validity period of the offer, the bidder shall be treated as ineligible for participation in the future tenders for a period of 6 months from the date of withdrawal of the bid, and also in re-tendering of this particular package.
+3. If it is established that the bidder/his representatives have committed any fraud while competing for this contract, the Employer shall be entitled to disqualify the Bidder(s)/Contractor(s) from the bidding process and forfeit the Earnest Money Deposit. Additionally, the Employer may exclude/blacklist the Bidder for any future tenders/contracts award process.
+4. If declarations given regarding debarment policy compliance are found to be incorrect subsequent to award of Contract, NTPC/Employer shall have the full right to terminate the Contract and take any action as per applicable laws for breach of contract including forfeiture of Bid Security/Performance Bank Guarantee.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Not Required</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>1 field(s): Assignment Fees</t>
+          <t>clean</t>
         </is>
       </c>
     </row>
@@ -669,42 +669,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Tender</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Final Value</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Source (file, page)</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Rules layer read</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>AI layer read</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Flag</t>
         </is>
@@ -723,7 +723,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+          <t>Tender Id 103392745 - Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+          <t>Tender Id 103392745 - Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -901,30 +901,38 @@
       <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>6. Assignment Fees</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND - verify manually</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Tender-Summary-103392745.pdf (p.3)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>not_found</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -939,16 +947,19 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>1. Only CPCB authorized Auditors shall undertake the compliance audit for ash disposal for NTPC Solapur as per MOEF&amp;CC notification dated 31.12.2021 and its subsequent amendments. (Bidder to submit documentary evidence in this regard, in absence of same Bids shall be liable for rejection.)
-2. The bidder should not be under any banning/suspension/withholding with NTPC Ltd.
-3. All the bidders have to submit the GTE template PAN, GSTIN and enlistment certificate issued OR copy of the email for this package sent by the buyer/tender inviting authority.
-4. MSE Purchase Preference: Purchase preference will be given to MSEs having valid Udyam Certificate and whose credentials are validated online through Udyam Registration portal. If L-1 is not an MSE and MSE Seller(s) has/have quoted price within L-1+ 15% of margin of purchase preference, such MSE Seller shall be given opportunity to match L-1 price and contract will be awarded for 100% of total value.
-5. EMD exemption for: IIMs/IITs/ NITs/ IISc./ CBRI/ CPRI/ GSI/CWPRS/ CWC/ NEERI/ CSIR Labs and other Govt. Institutes/agencies (excluding PSUs).</t>
+          <t>1. Minimum average annual turnover required: 51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
+2. OEM turnover requirement: NA.
+3. Financial years for preceding three (3) financial years: 2021-2022, 2020-2021, and 2019-2020.
+4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, as per Appendix-A to Attachment 3A2.
+5. Experience required (years and type): The bidder must be a LOCAL SUPPLIER. Specific years of experience are not explicitly mentioned, but past experience related to the scope of work is required as per Attachment 3 and 4. For MSEs, the experience requirement is also subject to "Udyam Registration" and "Major Activity" not being "TRADING".
+6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents for each Qualifying Requirement criteria.
+7. Exemptions from past performance requirements: NA.
+8. Exemptions for MS</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>210347177.pdf (p.5)</t>
+          <t>Tender-Summary-103392745.pdf (p.3)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1007,11 +1018,14 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>1. Only CPCB authorized Auditors shall undertake the compliance audit for ash disposal for NTPC Solapur as per MOEF&amp;CC notification dated 31.12.2021 and its subsequent amendments. (Bidder to submit documentary evidence in this regard, in absence of same Bids shall be liable for rejection.)
-2. The bidder should not be under any banning/suspension/withholding with NTPC Ltd.
-3. All the bidders have to submit the GTE template PAN, GSTIN and enlistment certificate issued OR copy of the email for this package sent by the buyer/tender inviting authority.
-4. MSE Purchase Preference: Purchase preference will be given to MSEs having valid Udyam Certificate and whose credentials are validated online through Udyam Registration portal. If L-1 is not an MSE and MSE Seller(s) has/have quoted price within L-1+ 15% of margin of purchase preference, such MSE Seller shall be given opportunity to match L-1 price and contract will be awarded for 100% of total value.
-5. EMD exemption for: IIMs/IITs/ NITs/ IISc./ CBRI/ CPRI/ GSI/CWPRS/ CWC/ NEERI/ CSIR Labs and other Govt. Institutes/agencies (excluding PSUs).</t>
+          <t>1. Minimum average annual turnover required: 51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
+2. OEM turnover requirement: NA.
+3. Financial years for preceding three (3) financial years: 2021-2022, 2020-2021, and 2019-2020.
+4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, as per Appendix-A to Attachment 3A2.
+5. Experience required (years and type): The bidder must be a LOCAL SUPPLIER. Specific years of experience are not explicitly mentioned, but past experience related to the scope of work is required as per Attachment 3 and 4. For MSEs, the experience requirement is also subject to "Udyam Registration" and "Major Activity" not being "TRADING".
+6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents for each Qualifying Requirement criteria.
+7. Exemptions from past performance requirements: NA.
+8. Exemptions for MS</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1094,12 +1108,15 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>LD: Applicable</t>
+          <t>1. If a bidder after having been issued the Notification of Award, either does not sign the Contract Agreement or does not submit an acceptable Performance Security, resulting in retendering, the bidder shall be treated ineligible for participation in re-tendering of this particular package and dealt as per the provisions of policy for Debarment from Business Dealings.
+2. If a bidder after opening of the tender withdraws its offer within the validity period of the offer, the bidder shall be treated as ineligible for participation in the future tenders for a period of 6 months from the date of withdrawal of the bid, and also in re-tendering of this particular package.
+3. If it is established that the bidder/his representatives have committed any fraud while competing for this contract, the Employer shall be entitled to disqualify the Bidder(s)/Contractor(s) from the bidding process and forfeit the Earnest Money Deposit. Additionally, the Employer may exclude/blacklist the Bidder for any future tenders/contracts award process.
+4. If declarations given regarding debarment policy compliance are found to be incorrect subsequent to award of Contract, NTPC/Employer shall have the full right to terminate the Contract and take any action as per applicable laws for breach of contract including forfeiture of Bid Security/Performance Bank Guarantee.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>210347180.pdf (p.5)</t>
+          <t>TENDER.pdf (p.23-24)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1138,7 +1155,10 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>LD: Applicable</t>
+          <t>1. If a bidder after having been issued the Notification of Award, either does not sign the Contract Agreement or does not submit an acceptable Performance Security, resulting in retendering, the bidder shall be treated ineligible for participation in re-tendering of this particular package and dealt as per the provisions of policy for Debarment from Business Dealings.
+2. If a bidder after opening of the tender withdraws its offer within the validity period of the offer, the bidder shall be treated as ineligible for participation in the future tenders for a period of 6 months from the date of withdrawal of the bid, and also in re-tendering of this particular package.
+3. If it is established that the bidder/his representatives have committed any fraud while competing for this contract, the Employer shall be entitled to disqualify the Bidder(s)/Contractor(s) from the bidding process and forfeit the Earnest Money Deposit. Additionally, the Employer may exclude/blacklist the Bidder for any future tenders/contracts award process.
+4. If declarations given regarding debarment policy compliance are found to be incorrect subsequent to award of Contract, NTPC/Employer shall have the full right to terminate the Contract and take any action as per applicable laws for breach of contract including forfeiture of Bid Security/Performance Bank Guarantee.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -1156,12 +1176,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Not Required</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>210347177.pdf (p.2)</t>
+          <t>Tender-Summary-103392745.pdf (p.2)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1176,7 +1196,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Not Required</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -1275,7 +1295,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>210347177.pdf (p.1)</t>
+          <t>Tender-Summary-103392745.pdf (p.1)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1317,259 +1337,259 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Tender</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Pages read</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Pages needing OCR</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>210347177.pdf</t>
         </is>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="5" t="inlineStr"/>
+      <c r="E2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>210347178.pdf</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="5" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>210347179.pdf</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="5" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>210347180.pdf</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="5" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>210347181.pdf</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="5" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>210347182.pdf</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="5" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>210347183.pdf</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="5" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>210347184.pdf</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="5" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>ATTACHMENT - 9 (2).pdf</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="5" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>ATTACHMENT - 9.pdf</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="5" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Tender-Summary-103392745.pdf</t>
         </is>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="5" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>TENDER.pdf</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="4" t="n">
         <v>417</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="5" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1590,132 +1610,132 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>How to read this workbook</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr"/>
+      <c r="B1" s="6" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Tender Summary</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>One row per tender folder, the 13 requested fields.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>For every field: the source file and page it came from, plus what each of the two independent readers (rules and AI) read. Use this to verify a value in seconds.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Documents Read</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Which files were opened, how many pages, how many needed OCR.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr"/>
-      <c r="B5" s="7" t="inlineStr"/>
+      <c r="A5" s="5" t="inlineStr"/>
+      <c r="B5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Cell colours</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
+      <c r="B6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Amber</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Needs your eye: the two readers disagreed, confidence was low, or the value came off a scanned page via OCR.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Not stated anywhere in the documents that were read.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr"/>
-      <c r="B9" s="7" t="inlineStr"/>
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Important</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>This tool eliminates the typing, not the review. Always confirm EMD, fees, and the submission deadline against the source page before acting on them.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Single reader</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Without a Gemini API key only the rules layer runs. Money and date fields are then capped at medium confidence and flagged, because nothing cross-checked them.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Percentages</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Security deposit and performance guarantees are normally a percentage of contract value, so that is what is reported. A rupee figure sitting next to a phrase like "up to" is a threshold, not the amount payable, and is flagged as such.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Excluded</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>WORKING FOLDER is skipped by design - it holds your own draft submissions, not the department's tender documents.</t>
         </is>

</xml_diff>

<commit_message>
Hide generic boilerplate documents from the AI completely
</commit_message>
<xml_diff>
--- a/Tender_Summary.xlsx
+++ b/Tender_Summary.xlsx
@@ -562,7 +562,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Tender Id 103392745 - Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+          <t>Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -572,7 +572,9 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
+          <t>Statutory audit of ash disposal for FY25-26
+[...]
+Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -593,28 +595,32 @@
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>1. Minimum average annual turnover required: 51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
-2. OEM turnover requirement: NA.
-3. Financial years for preceding three (3) financial years: 2021-2022, 2020-2021, and 2019-2020.
-4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, as per Appendix-A to Attachment 3A2.
+2. OEM turnover requirement: NA
+3. Financial years for Preceding three (3) financial years. The specific years are 2021-2022, 2020-2021, and 2019-2020.
+4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, is enclosed as per the format at Appendix-A to Attachment 3A2.
 5. Experience required (years and type): The bidder must be a LOCAL SUPPLIER. Specific years of experience are not explicitly mentioned, but past experience related to the scope of work is required as per Attachment 3 and 4. For MSEs, the experience requirement is also subject to "Udyam Registration" and "Major Activity" not being "TRADING".
-6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents for each Qualifying Requirement criteria.
-7. Exemptions from past performance requirements: NA.
-8. Exemptions for MSE / MSME / Start-ups: MSEs registered with appropriate bodies having UDYAM Registration for goods produced and services rendered are exempted from paying Earnest Money Deposit and are issued bid documents free of cost. MSE benefits are applicable for Service Contracts only, not for Works Contracts. Specific preference hierarchy for price band of L1 + 15% is outlined.
-9. Production capacity requirements: NA.
-10. Make in India requirements or preferences: Not Applicable. However, Class‑I local sup</t>
+6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents like Work Orders/Purchase Orders/Letter of Awards/Contract Agreement, client certificates etc. for each Qualifying Requirement criteria.
+7. Exemptions from past performance requirements: NA
+8. Exemptions for MSE / MSME / Start-ups: MSEs registered with District Industries Centres or Khadi and Village Industries Commission or Khadi and Village Industries Board or Coir Board or National Small Industries Corporation or Directorate of Handicrafts and Handloom or any other body specified by Ministry of Micro, Small and Medium Enterprises as per MSMED Act 2006, having</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under permitted uses/avenues, and comparison of this data with the information provided by the power plant in the annual compliance report. iii. Verification of the ash disposal into ash ponds data pertaining to the financial year (i.e. difference of ash generation and ash utilization, as above), and comparison of this data with the information provided by the power plant in the annual compliance report. iv. Assessment of total ash storage in operational and un-operation ash ponds and available storage capacity for further disposal at the end of financial year based on details and drawings of ash ponds provided by the power plant and ground verification of the information provided, and comparison of the storage and storage capacity with the information provided by the power plant in the annual compliance report. v. Assessment of ash slurry disposal and ash water re-circulation system used during the financial year, in respect ratio of water in the ash disposed to ash ponds, water used for ash slurry disposal to ash ponds, ash water recycled through AWRS, and ash water discharged into environment based on inspection of records provided by the power plant and ground verification, including the condition of surrounding environment in respect of ash released or breached, and comparison of the ground situat</t>
+          <t>Statutory audit of ash disposal for FY25-26. The bidder has to submit their offer inclusive of GST. The Service Provider hereby undertakes not to charge any money/fees/deductions in whatever manner, name, or form, or take any monetary/non-monetary considerations, or make any unlawful deductions from the compensation/salary of the manpower/employees/resources engaged by it and, to be deployed at the Buyer's site. The Service Provider further agrees that it will not indulge in any unethical practices and acknowledges that any non-compliance of the aforesaid undertaking will be treated as a material breach of the Contract, in which case the Buyer and GeM shall have the right to take appropriate independent actions including termination of the Contract and actions as per GeM Incident Management Policy.
+[...]
+Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under permitted uses/avenues, and comparison of this data with the information provided by the power plant in the annual compliance report. iii. Verification of the ash disposal into ash ponds data pertaining to the financial year (i.e. difference of ash generation and ash utilization, as above), and comparison of this data with the information provided by the power plant in the annual compliance report. iv. Assessment of total ash storage in operational and un-operation ash ponds and available stora</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>1. If a bidder after having been issued the Notification of Award, either does not sign the Contract Agreement or does not submit an acceptable Performance Security, resulting in retendering, the bidder shall be treated ineligible for participation in re-tendering of this particular package and dealt as per the provisions of policy for Debarment from Business Dealings.
-2. If a bidder after opening of the tender withdraws its offer within the validity period of the offer, the bidder shall be treated as ineligible for participation in the future tenders for a period of 6 months from the date of withdrawal of the bid, and also in re-tendering of this particular package.
-3. If it is established that the bidder/his representatives have committed any fraud while competing for this contract, the Employer shall be entitled to disqualify the Bidder(s)/Contractor(s) from the bidding process and forfeit the Earnest Money Deposit. Additionally, the Employer may exclude/blacklist the Bidder for any future tenders/contracts award process.
-4. If declarations given regarding debarment policy compliance are found to be incorrect subsequent to award of Contract, NTPC/Employer shall have the full right to terminate the Contract and take any action as per applicable laws for breach of contract including forfeiture of Bid Security/Performance Bank Guarantee.</t>
+          <t>LD: Applicable
+[...]
+1. Ineligibility for re-tendering: If a bidder/contractor is treated ineligible for participation in re-tendering of the package, they shall also be dealt as per provisions of policy for Debarment from Business Dealings.
+2. Withdrawal of Offer: If a bidder withdraws its offer within the validity period (where EMD is NIL/exempted), they shall be treated as ineligible for participation in future tenders for a period of 6 months from the date of withdrawal, and also in re-tendering of this particular package.
+3. Failure to Sign Contract/Submit Security: If a bidder does not sign the Contract Agreement or submit acceptable Performance Security resulting in re-tendering, they shall be treated ineligible for re-tendering and dealt as per Debarment policy.
+4. Fraud: If fraud is established, the bid shall be rejected. The Employer is entitled to exclude/blacklist the Bidder for any future tenders/contracts award process.
+[...]
+Liquidated Damages as per GCC clause-25.5.1</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -723,7 +729,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Tender Id 103392745 - Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+          <t>Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -743,7 +749,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Tender Id 103392745 - Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+          <t>Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -799,12 +805,14 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
+          <t>Statutory audit of ash disposal for FY25-26
+[...]
+Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>210347180.pdf (p.2)</t>
+          <t>Tender-Summary-103392745.pdf (p.1), 210347180.pdf (p.2)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -819,7 +827,9 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
+          <t>Statutory audit of ash disposal for FY25-26
+[...]
+Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -948,18 +958,16 @@
       <c r="C8" s="2" t="inlineStr">
         <is>
           <t>1. Minimum average annual turnover required: 51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
-2. OEM turnover requirement: NA.
-3. Financial years for preceding three (3) financial years: 2021-2022, 2020-2021, and 2019-2020.
-4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, as per Appendix-A to Attachment 3A2.
+2. OEM turnover requirement: NA
+3. Financial years for Preceding three (3) financial years. The specific years are 2021-2022, 2020-2021, and 2019-2020.
+4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, is enclosed as per the format at Appendix-A to Attachment 3A2.
 5. Experience required (years and type): The bidder must be a LOCAL SUPPLIER. Specific years of experience are not explicitly mentioned, but past experience related to the scope of work is required as per Attachment 3 and 4. For MSEs, the experience requirement is also subject to "Udyam Registration" and "Major Activity" not being "TRADING".
-6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents for each Qualifying Requirement criteria.
-7. Exemptions from past performance requirements: NA.
-8. Exemptions for MS</t>
+6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents like Work Orders/Purchase Orders/Letter of Awards/Contract Agreement</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Tender-Summary-103392745.pdf (p.3)</t>
+          <t>Tender-Summary-103392745.pdf (p.3), 210347177.pdf (p.5), 210347184.pdf (p.11-14)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1019,13 +1027,11 @@
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>1. Minimum average annual turnover required: 51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
-2. OEM turnover requirement: NA.
-3. Financial years for preceding three (3) financial years: 2021-2022, 2020-2021, and 2019-2020.
-4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, as per Appendix-A to Attachment 3A2.
+2. OEM turnover requirement: NA
+3. Financial years for Preceding three (3) financial years. The specific years are 2021-2022, 2020-2021, and 2019-2020.
+4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, is enclosed as per the format at Appendix-A to Attachment 3A2.
 5. Experience required (years and type): The bidder must be a LOCAL SUPPLIER. Specific years of experience are not explicitly mentioned, but past experience related to the scope of work is required as per Attachment 3 and 4. For MSEs, the experience requirement is also subject to "Udyam Registration" and "Major Activity" not being "TRADING".
-6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents for each Qualifying Requirement criteria.
-7. Exemptions from past performance requirements: NA.
-8. Exemptions for MS</t>
+6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents like Work Orders/Purchase Orders/Letter of Awards/Contract Agreement</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1043,17 +1049,19 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under permitted uses/avenues, and comparison of this data with the information provided by the power plant in the annual compliance report. iii. Verification of the ash disposal into ash ponds data pertaining to the financial year (i.e. difference of ash generation and ash utilization, as above), and comparison of this data with the information provided by the power plant in the annual compliance report. iv. Assessment of total ash storage in operational and un-operation ash ponds and available storage capacity for further disposal at the end of financial year based on details and drawings of ash ponds provided by the power plant and ground verification of the information provided, and comparison of the storage and storage capacity with the information provided by the power plant in the annual compliance report.</t>
+          <t>Statutory audit of ash disposal for FY25-26. The bidder has to submit their offer inclusive of GST. The Service Provider hereby undertakes not to charge any money/fees/deductions in whatever manner, name, or form, or take any monetary/non-monetary considerations, or make any unlawful deductions from the compensation/salary of the manpower/employees/resources engaged by it and, to be deployed at the Buyer's site. The Service Provider further agrees that it will not indulge in any unethical practices and acknowledges that any non-compliance of the aforesaid undertaking will be treated as a material breach of the Contract, in which case the Buyer and GeM shall have the right to take appropriate independent actions including termination of the Contract and actions as per GeM Incident Management Policy.
+[...]
+Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>210347180.pdf (p.3)</t>
+          <t>210347177.pdf (p.5), 210347180.pdf (p.3)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1090,7 +1098,9 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under permitted uses/avenues, and comparison of this data with the information provided by the power plant in the annual compliance report. iii. Verification of the ash disposal into ash ponds data pertaining to the financial year (i.e. difference of ash generation and ash utilization, as above), and comparison of this data with the information provided by the power plant in the annual compliance report. iv. Assessment of total ash storage in operational and un-operation ash ponds and available storage capacity for further disposal at the end of financial year based on details and drawings of ash ponds provided by the power plant and ground verification of the information provided, and comparison of the storage and storage capacity with the information provided by the power plant in the annual compliance report.</t>
+          <t>Statutory audit of ash disposal for FY25-26. The bidder has to submit their offer inclusive of GST. The Service Provider hereby undertakes not to charge any money/fees/deductions in whatever manner, name, or form, or take any monetary/non-monetary considerations, or make any unlawful deductions from the compensation/salary of the manpower/employees/resources engaged by it and, to be deployed at the Buyer's site. The Service Provider further agrees that it will not indulge in any unethical practices and acknowledges that any non-compliance of the aforesaid undertaking will be treated as a material breach of the Contract, in which case the Buyer and GeM shall have the right to take appropriate independent actions including termination of the Contract and actions as per GeM Incident Management Policy.
+[...]
+Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1108,15 +1118,19 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>1. If a bidder after having been issued the Notification of Award, either does not sign the Contract Agreement or does not submit an acceptable Performance Security, resulting in retendering, the bidder shall be treated ineligible for participation in re-tendering of this particular package and dealt as per the provisions of policy for Debarment from Business Dealings.
-2. If a bidder after opening of the tender withdraws its offer within the validity period of the offer, the bidder shall be treated as ineligible for participation in the future tenders for a period of 6 months from the date of withdrawal of the bid, and also in re-tendering of this particular package.
-3. If it is established that the bidder/his representatives have committed any fraud while competing for this contract, the Employer shall be entitled to disqualify the Bidder(s)/Contractor(s) from the bidding process and forfeit the Earnest Money Deposit. Additionally, the Employer may exclude/blacklist the Bidder for any future tenders/contracts award process.
-4. If declarations given regarding debarment policy compliance are found to be incorrect subsequent to award of Contract, NTPC/Employer shall have the full right to terminate the Contract and take any action as per applicable laws for breach of contract including forfeiture of Bid Security/Performance Bank Guarantee.</t>
+          <t>LD: Applicable
+[...]
+1. Ineligibility for re-tendering: If a bidder/contractor is treated ineligible for participation in re-tendering of the package, they shall also be dealt as per provisions of policy for Debarment from Business Dealings.
+2. Withdrawal of Offer: If a bidder withdraws its offer within the validity period (where EMD is NIL/exempted), they shall be treated as ineligible for participation in future tenders for a period of 6 months from the date of withdrawal, and also in re-tendering of this particular package.
+3. Failure to Sign Contract/Submit Security: If a bidder does not sign the Contract Agreement or submit acceptable Performance Security resulting in re-tendering, they shall be treated ineligible for re-tendering and dealt as per Debarment policy.
+4. Fraud: If fraud is established, the bid shall be rejected. The Employer is entitled to exclude/blacklist the Bidder for any future tenders/contracts award process.
+[...]
+Liquidated Damages as per GCC clause-25.5.1</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>TENDER.pdf (p.23-24)</t>
+          <t>210347180.pdf (p.5), 210347184.pdf (p.11), 210347184.pdf (p.22)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1155,10 +1169,14 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>1. If a bidder after having been issued the Notification of Award, either does not sign the Contract Agreement or does not submit an acceptable Performance Security, resulting in retendering, the bidder shall be treated ineligible for participation in re-tendering of this particular package and dealt as per the provisions of policy for Debarment from Business Dealings.
-2. If a bidder after opening of the tender withdraws its offer within the validity period of the offer, the bidder shall be treated as ineligible for participation in the future tenders for a period of 6 months from the date of withdrawal of the bid, and also in re-tendering of this particular package.
-3. If it is established that the bidder/his representatives have committed any fraud while competing for this contract, the Employer shall be entitled to disqualify the Bidder(s)/Contractor(s) from the bidding process and forfeit the Earnest Money Deposit. Additionally, the Employer may exclude/blacklist the Bidder for any future tenders/contracts award process.
-4. If declarations given regarding debarment policy compliance are found to be incorrect subsequent to award of Contract, NTPC/Employer shall have the full right to terminate the Contract and take any action as per applicable laws for breach of contract including forfeiture of Bid Security/Performance Bank Guarantee.</t>
+          <t>LD: Applicable
+[...]
+1. Ineligibility for re-tendering: If a bidder/contractor is treated ineligible for participation in re-tendering of the package, they shall also be dealt as per provisions of policy for Debarment from Business Dealings.
+2. Withdrawal of Offer: If a bidder withdraws its offer within the validity period (where EMD is NIL/exempted), they shall be treated as ineligible for participation in future tenders for a period of 6 months from the date of withdrawal, and also in re-tendering of this particular package.
+3. Failure to Sign Contract/Submit Security: If a bidder does not sign the Contract Agreement or submit acceptable Performance Security resulting in re-tendering, they shall be treated ineligible for re-tendering and dealt as per Debarment policy.
+4. Fraud: If fraud is established, the bid shall be rejected. The Employer is entitled to exclude/blacklist the Bidder for any future tenders/contracts award process.
+[...]
+Liquidated Damages as per GCC clause-25.5.1</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Sync latest CRM export changes to subdirectories
</commit_message>
<xml_diff>
--- a/Tender_Summary.xlsx
+++ b/Tender_Summary.xlsx
@@ -7,14 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tender Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRM Import" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents Read" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tender Summary'!$A$1:$O$2</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -457,200 +455,360 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:AY2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
-  </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tender Folder</t>
+          <t>Pipeline Id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>1. Tender Name</t>
+          <t>Pipeline Owner.id</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>2. Location / Address</t>
+          <t>Pipeline Owner</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>3. Purpose / Audit Type</t>
+          <t>Amount</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>4. Period</t>
+          <t>Pipeline Name</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>5. Tender Estimated Cost</t>
+          <t>Closing Date</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>6. Assignment Fees</t>
+          <t>Company Name.id</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>7. Eligibility Criteria</t>
+          <t>Company Name</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>8. Scope of Work</t>
+          <t>Stage</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>9. Penalty</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>10. Tender EMD</t>
+          <t>Lead Source</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>11. Tender SD</t>
+          <t>Contact Name.id</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>12. Tender Fees</t>
+          <t>Contact Name</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>13. Tender Submission Date</t>
+          <t>Created By.id</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Needs Review</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="150" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Modified By.id</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Modified By</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Created Time</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Modified Time</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Last Activity Time</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Layout.id</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Layout</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Record Creation Source ID</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Specific Reason for not Applying</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>EMD Amount</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>EMD Issuance Bank</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Details of EMD</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Date / Transfer of EMD</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Amount of Tender Fees</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Tech. Bid Opening</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Fin. Bid Opening</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>L1 - Information</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>L2 - Information</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>L3 - Information</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Tender No.</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>Date of Receiving of Tender Info.</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>City Name</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>Brief Reason for not applying</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>Tender Selection Method</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>Pre-Bid meeting</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>Date of Submission</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>Actual Submission Date</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>EMD Refund Status</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>Details of Dispatch</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>Our Quote</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>Due Date of Tender</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="100" customHeight="1">
+      <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+          <t>zcrm_1227282000000446001</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>1045-Solapur STPP, Solapur STPP, AT-FATATEWADI, PO-HOTGI STATION, SOUTH SOLAPUR, SOLAPUR, Maharashtra-413215</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Statutory audit of ash disposal for FY25-26
-[...]
-Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>1 Month</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Rs. 145,600</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>1. Minimum average annual turnover required: 51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
-2. OEM turnover requirement: NA
-3. Financial years for Preceding three (3) financial years. The specific years are 2021-2022, 2020-2021, and 2019-2020.
-4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, is enclosed as per the format at Appendix-A to Attachment 3A2.
-5. Experience required (years and type): The bidder must be a LOCAL SUPPLIER. Specific years of experience are not explicitly mentioned, but past experience related to the scope of work is required as per Attachment 3 and 4. For MSEs, the experience requirement is also subject to "Udyam Registration" and "Major Activity" not being "TRADING".
-6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents like Work Orders/Purchase Orders/Letter of Awards/Contract Agreement, client certificates etc. for each Qualifying Requirement criteria.
-7. Exemptions from past performance requirements: NA
-8. Exemptions for MSE / MSME / Start-ups: MSEs registered with District Industries Centres or Khadi and Village Industries Commission or Khadi and Village Industries Board or Coir Board or National Small Industries Corporation or Directorate of Handicrafts and Handloom or any other body specified by Ministry of Micro, Small and Medium Enterprises as per MSMED Act 2006, having</t>
-        </is>
-      </c>
+          <t>Vegad CA Tushar</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26. The bidder has to submit their offer inclusive of GST. The Service Provider hereby undertakes not to charge any money/fees/deductions in whatever manner, name, or form, or take any monetary/non-monetary considerations, or make any unlawful deductions from the compensation/salary of the manpower/employees/resources engaged by it and, to be deployed at the Buyer's site. The Service Provider further agrees that it will not indulge in any unethical practices and acknowledges that any non-compliance of the aforesaid undertaking will be treated as a material breach of the Contract, in which case the Buyer and GeM shall have the right to take appropriate independent actions including termination of the Contract and actions as per GeM Incident Management Policy.
-[...]
-Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under permitted uses/avenues, and comparison of this data with the information provided by the power plant in the annual compliance report. iii. Verification of the ash disposal into ash ponds data pertaining to the financial year (i.e. difference of ash generation and ash utilization, as above), and comparison of this data with the information provided by the power plant in the annual compliance report. iv. Assessment of total ash storage in operational and un-operation ash ponds and available stora</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>LD: Applicable
-[...]
-1. Ineligibility for re-tendering: If a bidder/contractor is treated ineligible for participation in re-tendering of the package, they shall also be dealt as per provisions of policy for Debarment from Business Dealings.
-2. Withdrawal of Offer: If a bidder withdraws its offer within the validity period (where EMD is NIL/exempted), they shall be treated as ineligible for participation in future tenders for a period of 6 months from the date of withdrawal, and also in re-tendering of this particular package.
-3. Failure to Sign Contract/Submit Security: If a bidder does not sign the Contract Agreement or submit acceptable Performance Security resulting in re-tendering, they shall be treated ineligible for re-tendering and dealt as per Debarment policy.
-4. Fraud: If fraud is established, the bid shall be rejected. The Employer is entitled to exclude/blacklist the Bidder for any future tenders/contracts award process.
-[...]
-Liquidated Damages as per GCC clause-25.5.1</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Not Applicable</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Not Applicable</t>
-        </is>
-      </c>
+          <t>Yet to Decide</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>25-08-2026 11:00:00</t>
+          <t>zcrm_1227282000000446001</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>clean</t>
-        </is>
-      </c>
+          <t>Vegad CA Tushar</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>zcrm_1227282000000446001</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Vegad CA Tushar</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>zcrm_1227282000000453106</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>Tenders</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr"/>
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
+          <t>Sales Pipeline Standard</t>
+        </is>
+      </c>
+      <c r="Z2" s="2" t="inlineStr"/>
+      <c r="AA2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AC2" s="2" t="inlineStr"/>
+      <c r="AD2" s="2" t="inlineStr"/>
+      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="AF2" s="2" t="inlineStr"/>
+      <c r="AG2" s="2" t="inlineStr"/>
+      <c r="AH2" s="2" t="inlineStr"/>
+      <c r="AI2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AK2" s="2" t="inlineStr"/>
+      <c r="AL2" s="2" t="inlineStr"/>
+      <c r="AM2" s="2" t="inlineStr"/>
+      <c r="AN2" s="2" t="inlineStr"/>
+      <c r="AO2" s="2" t="inlineStr"/>
+      <c r="AP2" s="2" t="inlineStr"/>
+      <c r="AQ2" s="2" t="inlineStr"/>
+      <c r="AR2" s="2" t="inlineStr"/>
+      <c r="AS2" s="2" t="inlineStr"/>
+      <c r="AT2" s="2" t="inlineStr"/>
+      <c r="AU2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AW2" s="2" t="inlineStr"/>
+      <c r="AX2" s="2" t="inlineStr"/>
+      <c r="AY2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -729,7 +887,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+          <t>Tender Id 103392745 - Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -749,7 +907,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+          <t>Tender Id 103392745 - Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -805,14 +963,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26
-[...]
-Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
+          <t>Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Tender-Summary-103392745.pdf (p.1), 210347180.pdf (p.2)</t>
+          <t>210347180.pdf (p.2)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -827,9 +983,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26
-[...]
-Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
+          <t>Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -885,12 +1039,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Rs. 145,600</t>
+          <t>₹ 145600.0</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Tender-Summary-103392745.pdf (p.2)</t>
+          <t>210347183.pdf (p.1)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -905,7 +1059,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Rs. 145,600</t>
+          <t>₹ 145600.0</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -928,7 +1082,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Tender-Summary-103392745.pdf (p.3)</t>
+          <t>210347177.pdf (p.1)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -957,17 +1111,14 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>1. Minimum average annual turnover required: 51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
-2. OEM turnover requirement: NA
-3. Financial years for Preceding three (3) financial years. The specific years are 2021-2022, 2020-2021, and 2019-2020.
-4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, is enclosed as per the format at Appendix-A to Attachment 3A2.
-5. Experience required (years and type): The bidder must be a LOCAL SUPPLIER. Specific years of experience are not explicitly mentioned, but past experience related to the scope of work is required as per Attachment 3 and 4. For MSEs, the experience requirement is also subject to "Udyam Registration" and "Major Activity" not being "TRADING".
-6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents like Work Orders/Purchase Orders/Letter of Awards/Contract Agreement</t>
+          <t>28.2 If a bidder after opening of tenders where EMD is ‘NIL/Not applicable’ or exempted for bidders as per policy guidelines, withdraws its offer within the validity period of the offer, then such bidder shall be treated as ineligible for participation in future tenders for a period of 6 months from the date of withdrawal of the bid, and also in re-tendering of this particular package.
+28.3 If a bidder after having been issued the Notification of Award/ Purchase Order of a package where EMD is ‘NIL/Not applicable’ or exempted for bidder as per policy guidelines, either does not sign the Contract Agreement pursuant to ITB Clause titled ‘Signing the Contract Agreement’ or does not submit an acceptable Performance Security pursuant to ITB Clause titled ‘Performance Security’, and which result in retendering of the package, then such bidder/contractor shall be treated ineligible for participation in re‑tendering of this particular package. Further, such bidder/contractor shall also be dealt as per the provisions of the contract and policy for Debarment from Business Dealings.
+29 ADHERENCE TO FRAUD PREVENTION POLICY (ITB Cl. 29.0) The Bidder along with its associate/ collaborators/ sub‑contractors/ sub‑vendors/ consultants/ service providers shall strictly adhere to the Fraud Prevention Policy of EMPLOYER displayed on its tender website http://www.ntpctender.com and shall immediately apprise Employer about any fraud or suspected fraud as soon as it comes to their notice. A certifi</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Tender-Summary-103392745.pdf (p.3), 210347177.pdf (p.5), 210347184.pdf (p.11-14)</t>
+          <t>210347184.pdf (p.11)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1026,12 +1177,9 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>1. Minimum average annual turnover required: 51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
-2. OEM turnover requirement: NA
-3. Financial years for Preceding three (3) financial years. The specific years are 2021-2022, 2020-2021, and 2019-2020.
-4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, is enclosed as per the format at Appendix-A to Attachment 3A2.
-5. Experience required (years and type): The bidder must be a LOCAL SUPPLIER. Specific years of experience are not explicitly mentioned, but past experience related to the scope of work is required as per Attachment 3 and 4. For MSEs, the experience requirement is also subject to "Udyam Registration" and "Major Activity" not being "TRADING".
-6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents like Work Orders/Purchase Orders/Letter of Awards/Contract Agreement</t>
+          <t>28.2 If a bidder after opening of tenders where EMD is ‘NIL/Not applicable’ or exempted for bidders as per policy guidelines, withdraws its offer within the validity period of the offer, then such bidder shall be treated as ineligible for participation in future tenders for a period of 6 months from the date of withdrawal of the bid, and also in re-tendering of this particular package.
+28.3 If a bidder after having been issued the Notification of Award/ Purchase Order of a package where EMD is ‘NIL/Not applicable’ or exempted for bidder as per policy guidelines, either does not sign the Contract Agreement pursuant to ITB Clause titled ‘Signing the Contract Agreement’ or does not submit an acceptable Performance Security pursuant to ITB Clause titled ‘Performance Security’, and which result in retendering of the package, then such bidder/contractor shall be treated ineligible for participation in re‑tendering of this particular package. Further, such bidder/contractor shall also be dealt as per the provisions of the contract and policy for Debarment from Business Dealings.
+29 ADHERENCE TO FRAUD PREVENTION POLICY (ITB Cl. 29.0) The Bidder along with its associate/ collaborators/ sub‑contractors/ sub‑vendors/ consultants/ service providers shall strictly adhere to the Fraud Prevention Policy of EMPLOYER displayed on its tender website http://www.ntpctender.com and shall immediately apprise Employer about any fraud or suspected fraud as soon as it comes to their notice. A certifi</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1049,19 +1197,17 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26. The bidder has to submit their offer inclusive of GST. The Service Provider hereby undertakes not to charge any money/fees/deductions in whatever manner, name, or form, or take any monetary/non-monetary considerations, or make any unlawful deductions from the compensation/salary of the manpower/employees/resources engaged by it and, to be deployed at the Buyer's site. The Service Provider further agrees that it will not indulge in any unethical practices and acknowledges that any non-compliance of the aforesaid undertaking will be treated as a material breach of the Contract, in which case the Buyer and GeM shall have the right to take appropriate independent actions including termination of the Contract and actions as per GeM Incident Management Policy.
-[...]
-Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under</t>
+          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under permitted uses/avenues, and comparison of this data with the information provided by the power plant in the annual compliance report. iii. Verification of the ash disposal into ash ponds data pertaining to the financial year (i.e. difference of ash generation and ash utilization, as above), and comparison of this data with the information provided by the power plant in the annual compliance report. iv. Assessment of total ash storage in operational and un-operation ash ponds and available storage capacity for further disposal at the end of financial year based on details and drawings of ash ponds provided by the power plant and ground verification of the information provided, and comparison of the storage and storage capacity with the information provided by the power plant in the annual compliance report.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>210347177.pdf (p.5), 210347180.pdf (p.3)</t>
+          <t>210347180.pdf (p.3)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1098,9 +1244,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26. The bidder has to submit their offer inclusive of GST. The Service Provider hereby undertakes not to charge any money/fees/deductions in whatever manner, name, or form, or take any monetary/non-monetary considerations, or make any unlawful deductions from the compensation/salary of the manpower/employees/resources engaged by it and, to be deployed at the Buyer's site. The Service Provider further agrees that it will not indulge in any unethical practices and acknowledges that any non-compliance of the aforesaid undertaking will be treated as a material breach of the Contract, in which case the Buyer and GeM shall have the right to take appropriate independent actions including termination of the Contract and actions as per GeM Incident Management Policy.
-[...]
-Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under</t>
+          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under permitted uses/avenues, and comparison of this data with the information provided by the power plant in the annual compliance report. iii. Verification of the ash disposal into ash ponds data pertaining to the financial year (i.e. difference of ash generation and ash utilization, as above), and comparison of this data with the information provided by the power plant in the annual compliance report. iv. Assessment of total ash storage in operational and un-operation ash ponds and available storage capacity for further disposal at the end of financial year based on details and drawings of ash ponds provided by the power plant and ground verification of the information provided, and comparison of the storage and storage capacity with the information provided by the power plant in the annual compliance report.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1118,19 +1262,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>LD: Applicable
-[...]
-1. Ineligibility for re-tendering: If a bidder/contractor is treated ineligible for participation in re-tendering of the package, they shall also be dealt as per provisions of policy for Debarment from Business Dealings.
-2. Withdrawal of Offer: If a bidder withdraws its offer within the validity period (where EMD is NIL/exempted), they shall be treated as ineligible for participation in future tenders for a period of 6 months from the date of withdrawal, and also in re-tendering of this particular package.
-3. Failure to Sign Contract/Submit Security: If a bidder does not sign the Contract Agreement or submit acceptable Performance Security resulting in re-tendering, they shall be treated ineligible for re-tendering and dealt as per Debarment policy.
-4. Fraud: If fraud is established, the bid shall be rejected. The Employer is entitled to exclude/blacklist the Bidder for any future tenders/contracts award process.
-[...]
-Liquidated Damages as per GCC clause-25.5.1</t>
+          <t>LD: Applicable</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>210347180.pdf (p.5), 210347184.pdf (p.11), 210347184.pdf (p.22)</t>
+          <t>210347180.pdf (p.5)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1169,14 +1306,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>LD: Applicable
-[...]
-1. Ineligibility for re-tendering: If a bidder/contractor is treated ineligible for participation in re-tendering of the package, they shall also be dealt as per provisions of policy for Debarment from Business Dealings.
-2. Withdrawal of Offer: If a bidder withdraws its offer within the validity period (where EMD is NIL/exempted), they shall be treated as ineligible for participation in future tenders for a period of 6 months from the date of withdrawal, and also in re-tendering of this particular package.
-3. Failure to Sign Contract/Submit Security: If a bidder does not sign the Contract Agreement or submit acceptable Performance Security resulting in re-tendering, they shall be treated ineligible for re-tendering and dealt as per Debarment policy.
-4. Fraud: If fraud is established, the bid shall be rejected. The Employer is entitled to exclude/blacklist the Bidder for any future tenders/contracts award process.
-[...]
-Liquidated Damages as per GCC clause-25.5.1</t>
+          <t>LD: Applicable</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -1194,12 +1324,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Not Required</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Tender-Summary-103392745.pdf (p.2)</t>
+          <t>210347177.pdf (p.2)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1214,7 +1344,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Not Required</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -1313,7 +1443,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Tender-Summary-103392745.pdf (p.1)</t>
+          <t>210347177.pdf (p.1)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Fix prose extraction accuracy by prioritizing the Rules Engine if it captured a much longer section than the AI
</commit_message>
<xml_diff>
--- a/Tender_Summary.xlsx
+++ b/Tender_Summary.xlsx
@@ -37,7 +37,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -85,6 +90,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -887,7 +895,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Tender Id 103392745 - Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+          <t>Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -907,7 +915,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Tender Id 103392745 - Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
+          <t>Custom Bid for Services - 200155534 Solapur AUD - Statutory audit of ash disposal for FY25-26</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -963,12 +971,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
+          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>210347180.pdf (p.2)</t>
+          <t>210347180.pdf (p.3)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -983,7 +991,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Annual Statutory Ash compliance audit at NTPC Solapur for FY25-26 in compliance to MOEFCC fly ash notification</t>
+          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1039,12 +1047,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>₹ 145600.0</t>
+          <t>Rs. 145,600</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>210347183.pdf (p.1)</t>
+          <t>Tender-Summary-103392745.pdf (p.2)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1059,7 +1067,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>₹ 145600.0</t>
+          <t>Rs. 145,600</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1082,7 +1090,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>210347177.pdf (p.1)</t>
+          <t>NOT FOUND (p.NOT FOUND)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1111,14 +1119,18 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>28.2 If a bidder after opening of tenders where EMD is ‘NIL/Not applicable’ or exempted for bidders as per policy guidelines, withdraws its offer within the validity period of the offer, then such bidder shall be treated as ineligible for participation in future tenders for a period of 6 months from the date of withdrawal of the bid, and also in re-tendering of this particular package.
-28.3 If a bidder after having been issued the Notification of Award/ Purchase Order of a package where EMD is ‘NIL/Not applicable’ or exempted for bidder as per policy guidelines, either does not sign the Contract Agreement pursuant to ITB Clause titled ‘Signing the Contract Agreement’ or does not submit an acceptable Performance Security pursuant to ITB Clause titled ‘Performance Security’, and which result in retendering of the package, then such bidder/contractor shall be treated ineligible for participation in re‑tendering of this particular package. Further, such bidder/contractor shall also be dealt as per the provisions of the contract and policy for Debarment from Business Dealings.
-29 ADHERENCE TO FRAUD PREVENTION POLICY (ITB Cl. 29.0) The Bidder along with its associate/ collaborators/ sub‑contractors/ sub‑vendors/ consultants/ service providers shall strictly adhere to the Fraud Prevention Policy of EMPLOYER displayed on its tender website http://www.ntpctender.com and shall immediately apprise Employer about any fraud or suspected fraud as soon as it comes to their notice. A certifi</t>
+          <t>Eligibility Criteria
+1. Minimum average annual turnover required: 51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
+2. OEM turnover requirement: NA
+3. Financial years for Preceding three (3) financial years. The specific years are 2021-2022, 2020-2021, and 2019-2020.
+4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, is enclosed as per the format at Appendix-A to Attachment 3A2.
+5. Experience required (years and type): The bidder must be a LOCAL SUPPLIER. Specific years of experience are not explicitly mentioned, but past experience related to the scope of work is required as per Attachment 3 and 4. For MSEs, the experience requirement is also subject to "Udyam Registration" and "Major Activity" not being "TRADING".
+6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents like Work Orders/Purchase Orders/Letter of Awar</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>210347184.pdf (p.11)</t>
+          <t>Tender-Summary-103392745.pdf (p.3-5)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1177,9 +1189,13 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>28.2 If a bidder after opening of tenders where EMD is ‘NIL/Not applicable’ or exempted for bidders as per policy guidelines, withdraws its offer within the validity period of the offer, then such bidder shall be treated as ineligible for participation in future tenders for a period of 6 months from the date of withdrawal of the bid, and also in re-tendering of this particular package.
-28.3 If a bidder after having been issued the Notification of Award/ Purchase Order of a package where EMD is ‘NIL/Not applicable’ or exempted for bidder as per policy guidelines, either does not sign the Contract Agreement pursuant to ITB Clause titled ‘Signing the Contract Agreement’ or does not submit an acceptable Performance Security pursuant to ITB Clause titled ‘Performance Security’, and which result in retendering of the package, then such bidder/contractor shall be treated ineligible for participation in re‑tendering of this particular package. Further, such bidder/contractor shall also be dealt as per the provisions of the contract and policy for Debarment from Business Dealings.
-29 ADHERENCE TO FRAUD PREVENTION POLICY (ITB Cl. 29.0) The Bidder along with its associate/ collaborators/ sub‑contractors/ sub‑vendors/ consultants/ service providers shall strictly adhere to the Fraud Prevention Policy of EMPLOYER displayed on its tender website http://www.ntpctender.com and shall immediately apprise Employer about any fraud or suspected fraud as soon as it comes to their notice. A certifi</t>
+          <t>Eligibility Criteria
+1. Minimum average annual turnover required: 51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
+2. OEM turnover requirement: NA
+3. Financial years for Preceding three (3) financial years. The specific years are 2021-2022, 2020-2021, and 2019-2020.
+4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, is enclosed as per the format at Appendix-A to Attachment 3A2.
+5. Experience required (years and type): The bidder must be a LOCAL SUPPLIER. Specific years of experience are not explicitly mentioned, but past experience related to the scope of work is required as per Attachment 3 and 4. For MSEs, the experience requirement is also subject to "Udyam Registration" and "Major Activity" not being "TRADING".
+6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents like Work Orders/Purchase Orders/Letter of Awar</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1197,17 +1213,17 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under permitted uses/avenues, and comparison of this data with the information provided by the power plant in the annual compliance report. iii. Verification of the ash disposal into ash ponds data pertaining to the financial year (i.e. difference of ash generation and ash utilization, as above), and comparison of this data with the information provided by the power plant in the annual compliance report. iv. Assessment of total ash storage in operational and un-operation ash ponds and available storage capacity for further disposal at the end of financial year based on details and drawings of ash ponds provided by the power plant and ground verification of the information provided, and comparison of the storage and storage capacity with the information provided by the power plant in the annual compliance report.</t>
+          <t>Statutory audit of ash disposal for FY25-26. The bidder has to submit their offer inclusive of GST. The Service Provider hereby undertakes not to charge any money/fees/deductions in whatever manner, name, or form, or take any monetary/non-monetary considerations, or make any unlawful deductions from the compensation/salary of the manpower/employees/resources engaged by it and, to be deployed at the Buyer's site. The Service Provider further agrees that it will not indulge in any unethical practices and acknowledges that any non-compliance of the aforesaid undertaking will be treated as a material breach of the Contract, in which case the Buyer and GeM shall have the right to take appropriate independent actions including termination of the Contract and actions as per GeM Incident Management Policy.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>210347180.pdf (p.3)</t>
+          <t>210347177.pdf (p.5)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1244,7 +1260,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard. The work involves: i. Verification of ash generation data pertaining to the financial year based on inspection of records of coal receipt/consumption and average ash content in coal, and comparison of this data with the information provided by the power plant in the annual compliance report. ii. Verification of fly ash and bottom ash utilization data pertaining to the financial year based on inspection of records of ash supplied to the user agencies covered under permitted uses/avenues, and comparison of this data with the information provided by the power plant in the annual compliance report. iii. Verification of the ash disposal into ash ponds data pertaining to the financial year (i.e. difference of ash generation and ash utilization, as above), and comparison of this data with the information provided by the power plant in the annual compliance report. iv. Assessment of total ash storage in operational and un-operation ash ponds and available storage capacity for further disposal at the end of financial year based on details and drawings of ash ponds provided by the power plant and ground verification of the information provided, and comparison of the storage and storage capacity with the information provided by the power plant in the annual compliance report.</t>
+          <t>Statutory audit of ash disposal for FY25-26. The bidder has to submit their offer inclusive of GST. The Service Provider hereby undertakes not to charge any money/fees/deductions in whatever manner, name, or form, or take any monetary/non-monetary considerations, or make any unlawful deductions from the compensation/salary of the manpower/employees/resources engaged by it and, to be deployed at the Buyer's site. The Service Provider further agrees that it will not indulge in any unethical practices and acknowledges that any non-compliance of the aforesaid undertaking will be treated as a material breach of the Contract, in which case the Buyer and GeM shall have the right to take appropriate independent actions including termination of the Contract and actions as per GeM Incident Management Policy.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1262,12 +1278,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>LD: Applicable</t>
+          <t>The Bid Security may be forfeited a. If the Bidder withdraws or varies its Bid during the period of Bid validity; b. If the Bidder does not accept the correction of its Bid Price pursuant to ITB Sub-Clause for Arithmetical Correction. c. If the Bidder refuses to withdraw, without any cost to the Employer, any deviation, variation, additional condition or any other mention anywhere in the bid (Price bid in case of Two Stage Bid), contrary to the provisions of bidding documents; d. In the case of a successful Bidder, if the Bidder fails within the specified time limit to furnish the required Contract Performance Guarantee/Security Deposit in accordance with relevant clause of ITB. e. If the bidder/his representatives commits any fraud while competing for this contract pursuant to Fraud Prevention Policy of NTPC. f. In case the Bidder/Contractor is disqualified from bidding process in terms of Section 3 and 4 of Integrity Pact (IF APPLICABLE). g. Any suppression of material fact or false declaration regarding Insolvency, bankruptcy and Liquidation proceeding against Bidder, Associate, Collaborator or Technology Provider</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>210347180.pdf (p.5)</t>
+          <t>210347184.pdf (p.6)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1306,7 +1322,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>LD: Applicable</t>
+          <t>The Bid Security may be forfeited a. If the Bidder withdraws or varies its Bid during the period of Bid validity; b. If the Bidder does not accept the correction of its Bid Price pursuant to ITB Sub-Clause for Arithmetical Correction. c. If the Bidder refuses to withdraw, without any cost to the Employer, any deviation, variation, additional condition or any other mention anywhere in the bid (Price bid in case of Two Stage Bid), contrary to the provisions of bidding documents; d. In the case of a successful Bidder, if the Bidder fails within the specified time limit to furnish the required Contract Performance Guarantee/Security Deposit in accordance with relevant clause of ITB. e. If the bidder/his representatives commits any fraud while competing for this contract pursuant to Fraud Prevention Policy of NTPC. f. In case the Bidder/Contractor is disqualified from bidding process in terms of Section 3 and 4 of Integrity Pact (IF APPLICABLE). g. Any suppression of material fact or false declaration regarding Insolvency, bankruptcy and Liquidation proceeding against Bidder, Associate, Collaborator or Technology Provider</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -1324,12 +1340,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Not Required</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>210347177.pdf (p.2)</t>
+          <t>Tender-Summary-103392745.pdf (p.2)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1344,48 +1360,52 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Not Required</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
     </row>
     <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>11. Tender SD</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>210347180.pdf (p.5)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>2.5% of contract value (for MSE‑SC/ST and/or MSE‑Women vendors)   [rules read: 5.0% of the total Contract Price]</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>210347178.pdf (p.2)</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>5.0% of the total Contract Price</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>2.5% of contract value (for MSE‑SC/ST and/or MSE‑Women vendors)</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>CHECK - readers disagree</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -1400,7 +1420,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Not Applicable at GeM Portal.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1420,7 +1440,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Not Applicable at GeM Portal.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -1443,7 +1463,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>210347177.pdf (p.1)</t>
+          <t>Tender-Summary-103392745.pdf (p.1)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1512,232 +1532,232 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>210347177.pdf</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="4" t="inlineStr"/>
+      <c r="E2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>210347178.pdf</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="4" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>210347179.pdf</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="4" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>210347180.pdf</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="4" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>210347181.pdf</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="4" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>210347182.pdf</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="4" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>210347183.pdf</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="4" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>210347184.pdf</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="4" t="inlineStr"/>
+      <c r="E9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>ATTACHMENT - 9 (2).pdf</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="4" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>ATTACHMENT - 9.pdf</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="4" t="inlineStr"/>
+      <c r="E11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Tender-Summary-103392745.pdf</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="4" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>docs</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>TENDER.pdf</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="5" t="n">
         <v>417</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="4" t="inlineStr"/>
+      <c r="E13" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1758,132 +1778,132 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>How to read this workbook</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr"/>
+      <c r="B1" s="7" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Tender Summary</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>One row per tender folder, the 13 requested fields.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>For every field: the source file and page it came from, plus what each of the two independent readers (rules and AI) read. Use this to verify a value in seconds.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Documents Read</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Which files were opened, how many pages, how many needed OCR.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr"/>
-      <c r="B5" s="6" t="inlineStr"/>
+      <c r="A5" s="6" t="inlineStr"/>
+      <c r="B5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Cell colours</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
+      <c r="B6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Amber</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Needs your eye: the two readers disagreed, confidence was low, or the value came off a scanned page via OCR.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Not stated anywhere in the documents that were read.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr"/>
-      <c r="B9" s="6" t="inlineStr"/>
+      <c r="A9" s="6" t="inlineStr"/>
+      <c r="B9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Important</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>This tool eliminates the typing, not the review. Always confirm EMD, fees, and the submission deadline against the source page before acting on them.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Single reader</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Without a Gemini API key only the rules layer runs. Money and date fields are then capped at medium confidence and flagged, because nothing cross-checked them.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Percentages</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Security deposit and performance guarantees are normally a percentage of contract value, so that is what is reported. A rupee figure sitting next to a phrase like "up to" is a threshold, not the amount payable, and is flagged as such.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Excluded</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>WORKING FOLDER is skipped by design - it holds your own draft submissions, not the department's tender documents.</t>
         </is>

</xml_diff>

<commit_message>
Fix final merge logic to prevent AI NOT FOUND from silencing the rules engine and strictly enforce prose length overrides
</commit_message>
<xml_diff>
--- a/Tender_Summary.xlsx
+++ b/Tender_Summary.xlsx
@@ -971,12 +971,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard.</t>
+          <t>Statutory audit of ash disposal for FY25-26</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>210347180.pdf (p.3)</t>
+          <t>210347177.pdf (p.1)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26 at site, preparation and submission of report to CPCB and other concerned authorities with a copy to NTPC Solapur in line with the CPCB SOP/Guidelines etc in this regard.</t>
+          <t>Statutory audit of ash disposal for FY25-26</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1085,23 +1085,23 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Rs. 1,10,000 per month (FY 2022-23)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND (p.NOT FOUND)</t>
+          <t>210347184.pdf (p.17)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Rs. 1,10,000 per month (FY 2022-23)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -1119,18 +1119,19 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Eligibility Criteria
-1. Minimum average annual turnover required: 51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
-2. OEM turnover requirement: NA
-3. Financial years for Preceding three (3) financial years. The specific years are 2021-2022, 2020-2021, and 2019-2020.
-4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, is enclosed as per the format at Appendix-A to Attachment 3A2.
-5. Experience required (years and type): The bidder must be a LOCAL SUPPLIER. Specific years of experience are not explicitly mentioned, but past experience related to the scope of work is required as per Attachment 3 and 4. For MSEs, the experience requirement is also subject to "Udyam Registration" and "Major Activity" not being "TRADING".
-6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents like Work Orders/Purchase Orders/Letter of Awar</t>
+          <t>1. The bidder should not be under any banning/suspension/withholding with NTPC Ltd. 
+2. Only CPCB authorized Auditors shall undertake the compliance audit for ash disposal for NTPC Solapur as per MOEF&amp;CC notification dated 31.12.2021 and its subsequent amendments. ( Bidder to submit documentary evidence in this regard, in absence of same Bids shall be liable for rejection.
+3. Bidders while participating in a bid should submit price element(s) in Financial bid only. Accordingly, all bidders are advised not to mention any price element(s) in the technical bid, else the offer shall be rejected as nonresponsive, except in case of Single Packet Bidding.
+4. All the bidders have to submit the GTE template PAN, GSTIN and enlistment certificate issued OR copy of the email for this package sent by the buyer/tender inviting authority.
+5. The bidder has to submit their offer inclusive of GST.
+6. The bidder has to mention GST % in the offer.
+7. Bidders may please note that GeM is capturing and showing the IP addresses used by the Buyer and the Bidder(s) /Seller(s). The received bids having matching/common IP address with either Bidder(s)/Seller(s) or Buyer, shall be outrightly rejected &amp; shall not be considered for further evaluation.
+8. The Service Provider hereby undertakes not to charge any money/fees/ deductions in whatever manner, name, or form, or take any monetary/non-monetary considerations, or make any unlawful deductions from the compensation/salary of the manpower/employees/res</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Tender-Summary-103392745.pdf (p.3-5)</t>
+          <t>210347177.pdf (p.5)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1189,13 +1190,14 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Eligibility Criteria
-1. Minimum average annual turnover required: 51 Lakhs (Rs. Fifty one Lakh only) or equivalent foreign currency.
-2. OEM turnover requirement: NA
-3. Financial years for Preceding three (3) financial years. The specific years are 2021-2022, 2020-2021, and 2019-2020.
-4. Documents required to prove turnover: Audited financial statements for the last 3 financial years. If audited results for the last preceding financial year are not available, a certification of financial statement from a practicing chartered accountant. Certificate from the CEO/CFO of the Holding Company stating that the unaudited unconsolidated financial statements form part of the consolidated financial statements of the Holding Company, is enclosed as per the format at Appendix-A to Attachment 3A2.
-5. Experience required (years and type): The bidder must be a LOCAL SUPPLIER. Specific years of experience are not explicitly mentioned, but past experience related to the scope of work is required as per Attachment 3 and 4. For MSEs, the experience requirement is also subject to "Udyam Registration" and "Major Activity" not being "TRADING".
-6. Past performance / similar work experience: Details of past experience, such as authentic Work Orders/ Purchase Orders/ Letter of Awards/ Contract Agreements, and client certificates, completion certificate, etc., are required. Bidder is not permitted to quote more than 3 (three) times the reference documents like Work Orders/Purchase Orders/Letter of Awar</t>
+          <t>1. The bidder should not be under any banning/suspension/withholding with NTPC Ltd. 
+2. Only CPCB authorized Auditors shall undertake the compliance audit for ash disposal for NTPC Solapur as per MOEF&amp;CC notification dated 31.12.2021 and its subsequent amendments. ( Bidder to submit documentary evidence in this regard, in absence of same Bids shall be liable for rejection.
+3. Bidders while participating in a bid should submit price element(s) in Financial bid only. Accordingly, all bidders are advised not to mention any price element(s) in the technical bid, else the offer shall be rejected as nonresponsive, except in case of Single Packet Bidding.
+4. All the bidders have to submit the GTE template PAN, GSTIN and enlistment certificate issued OR copy of the email for this package sent by the buyer/tender inviting authority.
+5. The bidder has to submit their offer inclusive of GST.
+6. The bidder has to mention GST % in the offer.
+7. Bidders may please note that GeM is capturing and showing the IP addresses used by the Buyer and the Bidder(s) /Seller(s). The received bids having matching/common IP address with either Bidder(s)/Seller(s) or Buyer, shall be outrightly rejected &amp; shall not be considered for further evaluation.
+8. The Service Provider hereby undertakes not to charge any money/fees/ deductions in whatever manner, name, or form, or take any monetary/non-monetary considerations, or make any unlawful deductions from the compensation/salary of the manpower/employees/res</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1213,17 +1215,17 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26. The bidder has to submit their offer inclusive of GST. The Service Provider hereby undertakes not to charge any money/fees/deductions in whatever manner, name, or form, or take any monetary/non-monetary considerations, or make any unlawful deductions from the compensation/salary of the manpower/employees/resources engaged by it and, to be deployed at the Buyer's site. The Service Provider further agrees that it will not indulge in any unethical practices and acknowledges that any non-compliance of the aforesaid undertaking will be treated as a material breach of the Contract, in which case the Buyer and GeM shall have the right to take appropriate independent actions including termination of the Contract and actions as per GeM Incident Management Policy.</t>
+          <t>May please refer Section V of Bidding Documents.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>210347177.pdf (p.5)</t>
+          <t>210347179.pdf (p.3)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1260,7 +1262,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Statutory audit of ash disposal for FY25-26. The bidder has to submit their offer inclusive of GST. The Service Provider hereby undertakes not to charge any money/fees/deductions in whatever manner, name, or form, or take any monetary/non-monetary considerations, or make any unlawful deductions from the compensation/salary of the manpower/employees/resources engaged by it and, to be deployed at the Buyer's site. The Service Provider further agrees that it will not indulge in any unethical practices and acknowledges that any non-compliance of the aforesaid undertaking will be treated as a material breach of the Contract, in which case the Buyer and GeM shall have the right to take appropriate independent actions including termination of the Contract and actions as per GeM Incident Management Policy.</t>
+          <t>May please refer Section V of Bidding Documents.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1278,12 +1280,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>The Bid Security may be forfeited a. If the Bidder withdraws or varies its Bid during the period of Bid validity; b. If the Bidder does not accept the correction of its Bid Price pursuant to ITB Sub-Clause for Arithmetical Correction. c. If the Bidder refuses to withdraw, without any cost to the Employer, any deviation, variation, additional condition or any other mention anywhere in the bid (Price bid in case of Two Stage Bid), contrary to the provisions of bidding documents; d. In the case of a successful Bidder, if the Bidder fails within the specified time limit to furnish the required Contract Performance Guarantee/Security Deposit in accordance with relevant clause of ITB. e. If the bidder/his representatives commits any fraud while competing for this contract pursuant to Fraud Prevention Policy of NTPC. f. In case the Bidder/Contractor is disqualified from bidding process in terms of Section 3 and 4 of Integrity Pact (IF APPLICABLE). g. Any suppression of material fact or false declaration regarding Insolvency, bankruptcy and Liquidation proceeding against Bidder, Associate, Collaborator or Technology Provider</t>
+          <t>59. Liquidated Damages GCC clause-25.5.1 As per GCC</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>210347184.pdf (p.6)</t>
+          <t>210347184.pdf (p.22)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1322,7 +1324,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>The Bid Security may be forfeited a. If the Bidder withdraws or varies its Bid during the period of Bid validity; b. If the Bidder does not accept the correction of its Bid Price pursuant to ITB Sub-Clause for Arithmetical Correction. c. If the Bidder refuses to withdraw, without any cost to the Employer, any deviation, variation, additional condition or any other mention anywhere in the bid (Price bid in case of Two Stage Bid), contrary to the provisions of bidding documents; d. In the case of a successful Bidder, if the Bidder fails within the specified time limit to furnish the required Contract Performance Guarantee/Security Deposit in accordance with relevant clause of ITB. e. If the bidder/his representatives commits any fraud while competing for this contract pursuant to Fraud Prevention Policy of NTPC. f. In case the Bidder/Contractor is disqualified from bidding process in terms of Section 3 and 4 of Integrity Pact (IF APPLICABLE). g. Any suppression of material fact or false declaration regarding Insolvency, bankruptcy and Liquidation proceeding against Bidder, Associate, Collaborator or Technology Provider</t>
+          <t>59. Liquidated Damages GCC clause-25.5.1 As per GCC</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -1340,12 +1342,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Required: No</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Tender-Summary-103392745.pdf (p.2)</t>
+          <t>210347177.pdf (p.2)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1360,7 +1362,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Required: No</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -1378,12 +1380,12 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>2.5% of contract value (for MSE‑SC/ST and/or MSE‑Women vendors)   [rules read: 5.0% of the total Contract Price]</t>
+          <t>ePBG Required: No. Performance Bank Guarantee shall be 2.5% of contract value in place of original 5% of contract value for all MSE-SC/ST and/or MSE- Women vendors on whom order is placed.   [rules read: 5.0% of the total Contract Price]</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>210347178.pdf (p.2)</t>
+          <t>210347177.pdf (p.6)</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1398,7 +1400,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>2.5% of contract value (for MSE‑SC/ST and/or MSE‑Women vendors)</t>
+          <t>ePBG Required: No. Performance Bank Guarantee shall be 2.5% of contract value in place of original 5% of contract value for all MSE-SC/ST and/or MSE- Women vendors on whom order is placed.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1463,7 +1465,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Tender-Summary-103392745.pdf (p.1)</t>
+          <t>210347177.pdf (p.1)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">

</xml_diff>